<commit_message>
Actualización de datos en mongo dinamicamente
</commit_message>
<xml_diff>
--- a/Morosos/informe_cartas_y_juntas.xlsx
+++ b/Morosos/informe_cartas_y_juntas.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="695" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1311" uniqueCount="378">
   <si>
     <t>dia_cita</t>
   </si>
@@ -55,22 +55,28 @@
     <t>pensiones pendientes</t>
   </si>
   <si>
-    <t>25</t>
-  </si>
-  <si>
-    <t>julio</t>
+    <t>06</t>
+  </si>
+  <si>
+    <t>sep</t>
   </si>
   <si>
     <t>Liliana María García Marín</t>
   </si>
   <si>
-    <t>21 julio de 2026</t>
-  </si>
-  <si>
-    <t>Biblioteca</t>
-  </si>
-  <si>
-    <t>7 am</t>
+    <t>1 septiembre de 2026</t>
+  </si>
+  <si>
+    <t>b</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>Alvarez Teran Josue</t>
+  </si>
+  <si>
+    <t>Alvarez Valencia Ana Elisa</t>
   </si>
   <si>
     <t>Alzate Monsalve David</t>
@@ -82,30 +88,72 @@
     <t>Arango Salazar Ximena</t>
   </si>
   <si>
+    <t>Arbelaez Torres Maksimilian</t>
+  </si>
+  <si>
     <t>Arenas Calderon Evoleth</t>
   </si>
   <si>
     <t>Arenas Calderon Salomon</t>
   </si>
   <si>
+    <t>Arias Valencia Violet</t>
+  </si>
+  <si>
     <t>Artunduaga Burgos Emmanuel</t>
   </si>
   <si>
     <t>Artunduaga Burgos Isaac</t>
   </si>
   <si>
-    <t>Artunduaga Burgos Sarahy</t>
-  </si>
-  <si>
-    <t>Cardona Mosquera Isaac</t>
+    <t>Atehortua Quintero Miguel Angel</t>
+  </si>
+  <si>
+    <t>Atehortua Quintero Simon</t>
+  </si>
+  <si>
+    <t>Bedoya Arevalo Estefany</t>
+  </si>
+  <si>
+    <t>Betancur Ortiz Isabella</t>
+  </si>
+  <si>
+    <t>Blandon Barragan Juan David</t>
+  </si>
+  <si>
+    <t>Bran Arrieta Saray</t>
+  </si>
+  <si>
+    <t>Buitrago Caicedo Juan Sebastian</t>
   </si>
   <si>
     <t>Cardona Mosquera Roxana</t>
   </si>
   <si>
+    <t>Carmona Taborda Luciana</t>
+  </si>
+  <si>
+    <t>Castaño Patiño Juan Jose</t>
+  </si>
+  <si>
+    <t>Castaño Viloria Sara</t>
+  </si>
+  <si>
     <t>Chavarria Osorio Luna Celeste</t>
   </si>
   <si>
+    <t>Chaverra Gomez Rebeca</t>
+  </si>
+  <si>
+    <t>Clavijo Quiceno Sara</t>
+  </si>
+  <si>
+    <t>Correa Castañeda Laura</t>
+  </si>
+  <si>
+    <t>Correa Castaño Christopher</t>
+  </si>
+  <si>
     <t>Cortes Correa Rebeca</t>
   </si>
   <si>
@@ -115,79 +163,157 @@
     <t>Cuervo Consuegra Tamara</t>
   </si>
   <si>
+    <t>De Luquez Bernal Mabel Sarai</t>
+  </si>
+  <si>
     <t>Diaz Gonzalez Matias</t>
   </si>
   <si>
     <t>Echeverri Agudelo Samuel</t>
   </si>
   <si>
-    <t>Garcia Ramirez Nicolas</t>
+    <t>Escalante Martinez Samuel</t>
+  </si>
+  <si>
+    <t>Florez Alvarez Juan David</t>
+  </si>
+  <si>
+    <t>Garcia Correa Andres Esteban</t>
+  </si>
+  <si>
+    <t>Garcia Gonzalez Juan Manuel</t>
   </si>
   <si>
     <t>Garcia Ramirez Thomás</t>
   </si>
   <si>
+    <t>Garzon Moreno Cristian</t>
+  </si>
+  <si>
+    <t>Gaviria Cespedes Brenda</t>
+  </si>
+  <si>
+    <t>Gaviria Cespedes Evelyn</t>
+  </si>
+  <si>
+    <t>Gil Arroyo David</t>
+  </si>
+  <si>
+    <t>Giraldo Avendaño Samuel</t>
+  </si>
+  <si>
+    <t>Giraldo Lozano Emma</t>
+  </si>
+  <si>
+    <t>Gomez Buitrago Mariangel</t>
+  </si>
+  <si>
+    <t>Gonzalez Bedoya Gracia</t>
+  </si>
+  <si>
+    <t>Gonzalez Bedoya Juanita</t>
+  </si>
+  <si>
+    <t>Gonzalez Gamboa Julieta</t>
+  </si>
+  <si>
     <t>Guette Ortiz Ashley Carolina</t>
   </si>
   <si>
-    <t>Guette Ortiz Norah Isabella</t>
+    <t>Henao Pinilla Simon</t>
+  </si>
+  <si>
+    <t>Hurtado Hurtado Sara</t>
   </si>
   <si>
     <t>Jaramillo Agudelo Ana Sofia</t>
   </si>
   <si>
+    <t>Londoño Sanchez Antonia</t>
+  </si>
+  <si>
     <t>Luna Rincon Juan Sebastian</t>
   </si>
   <si>
     <t>Machado Taborda Mateo</t>
   </si>
   <si>
+    <t>Mancera Londoño Josúe</t>
+  </si>
+  <si>
     <t>Manco Fonnegra Samuel</t>
   </si>
   <si>
     <t>Marin Vergara Nicolas</t>
   </si>
   <si>
-    <t>Martinez Alvarez Thiago</t>
-  </si>
-  <si>
-    <t>Martinez Ciro Josue</t>
+    <t>Marquez Mora Emilia</t>
   </si>
   <si>
     <t>Martinez Correa Tomas</t>
   </si>
   <si>
-    <t>Mesa Cardona Mariangel</t>
-  </si>
-  <si>
-    <t>Montoya Crumb Ahavah Joy</t>
-  </si>
-  <si>
-    <t>Montoya Crumb Aviva Faith</t>
-  </si>
-  <si>
-    <t>Montoya Crumb Samuel Robert</t>
+    <t>Monroy Garcia Sharon Yissel</t>
+  </si>
+  <si>
+    <t>Munive Echeverri Ariadna</t>
   </si>
   <si>
     <t>Muñoz Vellojin Mateo</t>
   </si>
   <si>
+    <t>Orrego Jimenez Analucia</t>
+  </si>
+  <si>
     <t>Ortega Zabala Abigail</t>
   </si>
   <si>
     <t>Ortiz Cano Sara</t>
   </si>
   <si>
+    <t>Ortiz Monsalve Sebastian</t>
+  </si>
+  <si>
+    <t>Ospina Cifuentes Antonella</t>
+  </si>
+  <si>
+    <t>Ospina Perez Samuel</t>
+  </si>
+  <si>
+    <t>Ospina Tuberquia Miguel Angel</t>
+  </si>
+  <si>
     <t>Perez Pino Susana</t>
   </si>
   <si>
+    <t>Peña González Sophia</t>
+  </si>
+  <si>
+    <t>Pinzon Rios Luna</t>
+  </si>
+  <si>
+    <t>Prieto Albán Isaac</t>
+  </si>
+  <si>
+    <t>Puerta Vanegas Isabel</t>
+  </si>
+  <si>
     <t>Pérez Hernández Salomé</t>
   </si>
   <si>
     <t>Ramirez Avila Daniel</t>
   </si>
   <si>
-    <t>Ramirez Avila Sara</t>
+    <t>Ramirez Morales Salome</t>
+  </si>
+  <si>
+    <t>Ramirez Pinzón Jeronimo</t>
+  </si>
+  <si>
+    <t>Restrepo Cadavid Emanuel</t>
+  </si>
+  <si>
+    <t>Restrepo Cadavid Isabela</t>
   </si>
   <si>
     <t>Restrepo Cortes Isabella</t>
@@ -202,6 +328,12 @@
     <t>Rizo Paez Elisa Victoria</t>
   </si>
   <si>
+    <t>Rojas Jimenez Sofia</t>
+  </si>
+  <si>
+    <t>Rueda Alvarez Josue</t>
+  </si>
+  <si>
     <t>Ruiz Aristizabal Nicolas</t>
   </si>
   <si>
@@ -226,19 +358,37 @@
     <t>Sanchez Justiniano Jose David</t>
   </si>
   <si>
+    <t>Sanchez Otalvaro Guadalupe</t>
+  </si>
+  <si>
+    <t>Sauls Peña Joshua</t>
+  </si>
+  <si>
     <t>Sayago Acevedo Isabella</t>
   </si>
   <si>
     <t>Sayago Acevedo Samuel</t>
   </si>
   <si>
+    <t>Segura Rios Emmanuel David</t>
+  </si>
+  <si>
     <t>Segura Rios Samuel Felipe</t>
   </si>
   <si>
     <t>Serna Ramirez Luciana</t>
   </si>
   <si>
-    <t>Sierra Peñaranda Miguel Angel</t>
+    <t>Sorza Hernandez Juan Martin</t>
+  </si>
+  <si>
+    <t>Suescun Yepes Juan Manuel</t>
+  </si>
+  <si>
+    <t>Suescun Yepes Luciana</t>
+  </si>
+  <si>
+    <t>Tabares Martinez Martina</t>
   </si>
   <si>
     <t>Tenorio Maya Liam</t>
@@ -247,18 +397,42 @@
     <t>Troya Rendon Emanuel</t>
   </si>
   <si>
+    <t>Usma Jaramillo Maria Celeste</t>
+  </si>
+  <si>
+    <t>Usuga Hidalgo Juan Sebastian</t>
+  </si>
+  <si>
     <t>Vanegas Pulgarin Sheray</t>
   </si>
   <si>
-    <t>Vasquez Rodas Josue</t>
+    <t>Vargas Wilches Maria Jose</t>
   </si>
   <si>
     <t>Velez Ortiz Simon</t>
   </si>
   <si>
+    <t>Villegas Vargas Mariangel</t>
+  </si>
+  <si>
+    <t>Zambrano Blanco Luis Felipe</t>
+  </si>
+  <si>
+    <t>Zapata Becerra Elizabeth</t>
+  </si>
+  <si>
     <t>Zapata Echeverry Abigail</t>
   </si>
   <si>
+    <t>Zorrilla Jaramillo Santiago</t>
+  </si>
+  <si>
+    <t>1015194657</t>
+  </si>
+  <si>
+    <t>1020309249</t>
+  </si>
+  <si>
     <t>1036521142</t>
   </si>
   <si>
@@ -268,30 +442,72 @@
     <t>1035424821</t>
   </si>
   <si>
+    <t>1021940719</t>
+  </si>
+  <si>
     <t>1020229348</t>
   </si>
   <si>
     <t>1011519538</t>
   </si>
   <si>
+    <t>1020125747</t>
+  </si>
+  <si>
     <t>1020322501</t>
   </si>
   <si>
     <t>1020327607</t>
   </si>
   <si>
-    <t>1020317655</t>
-  </si>
-  <si>
-    <t>1013464926</t>
+    <t>1011410509</t>
+  </si>
+  <si>
+    <t>1020235465</t>
+  </si>
+  <si>
+    <t>1036954386</t>
+  </si>
+  <si>
+    <t>1035006417</t>
+  </si>
+  <si>
+    <t>1235255951</t>
+  </si>
+  <si>
+    <t>1033198496</t>
+  </si>
+  <si>
+    <t>1011412659</t>
   </si>
   <si>
     <t>1013466654</t>
   </si>
   <si>
+    <t>1033198814</t>
+  </si>
+  <si>
+    <t>1023165980</t>
+  </si>
+  <si>
+    <t>1011514095</t>
+  </si>
+  <si>
     <t>1013358746</t>
   </si>
   <si>
+    <t>1020323596</t>
+  </si>
+  <si>
+    <t>1021935485</t>
+  </si>
+  <si>
+    <t>1025659461</t>
+  </si>
+  <si>
+    <t>1033192943</t>
+  </si>
+  <si>
     <t>1025898446</t>
   </si>
   <si>
@@ -301,79 +517,157 @@
     <t>1035003747</t>
   </si>
   <si>
+    <t>1202213225</t>
+  </si>
+  <si>
     <t>1021930204</t>
   </si>
   <si>
     <t>1011515086</t>
   </si>
   <si>
-    <t>1013353521</t>
+    <t>1038872200</t>
+  </si>
+  <si>
+    <t>1023554520</t>
+  </si>
+  <si>
+    <t>1018254177</t>
+  </si>
+  <si>
+    <t>1018252964</t>
   </si>
   <si>
     <t>1013362371</t>
   </si>
   <si>
+    <t>1020227383</t>
+  </si>
+  <si>
+    <t>1013349020</t>
+  </si>
+  <si>
+    <t>1013366022</t>
+  </si>
+  <si>
+    <t>1011517901</t>
+  </si>
+  <si>
+    <t>1037888238</t>
+  </si>
+  <si>
+    <t>1011517846</t>
+  </si>
+  <si>
+    <t>1018248214</t>
+  </si>
+  <si>
+    <t>1020228417</t>
+  </si>
+  <si>
+    <t>1020226198</t>
+  </si>
+  <si>
+    <t>1020321633</t>
+  </si>
+  <si>
     <t>1042587012</t>
   </si>
   <si>
-    <t>1018269052</t>
+    <t>1013364053</t>
+  </si>
+  <si>
+    <t>1025902964</t>
   </si>
   <si>
     <t>1041634370</t>
   </si>
   <si>
+    <t>1018254830</t>
+  </si>
+  <si>
     <t>1013350043</t>
   </si>
   <si>
     <t>1021931357</t>
   </si>
   <si>
+    <t>1097132180</t>
+  </si>
+  <si>
     <t>1020308169</t>
   </si>
   <si>
     <t>1018271477</t>
   </si>
   <si>
-    <t>1025899613</t>
-  </si>
-  <si>
-    <t>1035005666</t>
+    <t>1192469448</t>
   </si>
   <si>
     <t>1020225476</t>
   </si>
   <si>
-    <t>1025770324</t>
-  </si>
-  <si>
-    <t>1025776867</t>
-  </si>
-  <si>
-    <t>1013377365</t>
-  </si>
-  <si>
-    <t>1013370057</t>
+    <t>1038874283</t>
+  </si>
+  <si>
+    <t>1192465340</t>
   </si>
   <si>
     <t>1020307672</t>
   </si>
   <si>
+    <t>1011519079</t>
+  </si>
+  <si>
     <t>1011518615</t>
   </si>
   <si>
     <t>1020239882</t>
   </si>
   <si>
+    <t>1022150058</t>
+  </si>
+  <si>
+    <t>1011518603</t>
+  </si>
+  <si>
+    <t>1127538440</t>
+  </si>
+  <si>
+    <t>1038871132</t>
+  </si>
+  <si>
     <t>1020323103</t>
   </si>
   <si>
+    <t>1018261585</t>
+  </si>
+  <si>
+    <t>1056133411</t>
+  </si>
+  <si>
+    <t>1027664379</t>
+  </si>
+  <si>
+    <t>1020228568</t>
+  </si>
+  <si>
     <t>1020312315</t>
   </si>
   <si>
     <t>1020226915</t>
   </si>
   <si>
-    <t>1016601695</t>
+    <t>1023641253</t>
+  </si>
+  <si>
+    <t>1020239311</t>
+  </si>
+  <si>
+    <t>1195213635</t>
+  </si>
+  <si>
+    <t>1025656333</t>
   </si>
   <si>
     <t>1015079466</t>
@@ -388,6 +682,12 @@
     <t>1018273200</t>
   </si>
   <si>
+    <t>1021941636</t>
+  </si>
+  <si>
+    <t>1035011673</t>
+  </si>
+  <si>
     <t>1025895823</t>
   </si>
   <si>
@@ -412,19 +712,37 @@
     <t>1025904957</t>
   </si>
   <si>
+    <t>1020231885</t>
+  </si>
+  <si>
+    <t>1219213288</t>
+  </si>
+  <si>
     <t>1018271176</t>
   </si>
   <si>
     <t>1018254757</t>
   </si>
   <si>
+    <t>1141722491</t>
+  </si>
+  <si>
     <t>1141719278</t>
   </si>
   <si>
     <t>1035978921</t>
   </si>
   <si>
-    <t>1092540648</t>
+    <t>1069762747</t>
+  </si>
+  <si>
+    <t>1020228682</t>
+  </si>
+  <si>
+    <t>1023638076</t>
+  </si>
+  <si>
+    <t>1023595113</t>
   </si>
   <si>
     <t>1084474489</t>
@@ -433,111 +751,267 @@
     <t>1025667898</t>
   </si>
   <si>
+    <t>1033200952</t>
+  </si>
+  <si>
+    <t>1033190800</t>
+  </si>
+  <si>
     <t>1034925183</t>
   </si>
   <si>
-    <t>1034924450</t>
+    <t>1021929142</t>
   </si>
   <si>
     <t>1025900606</t>
   </si>
   <si>
+    <t>1021929216</t>
+  </si>
+  <si>
+    <t>1205964537</t>
+  </si>
+  <si>
+    <t>1021939636</t>
+  </si>
+  <si>
     <t>1023655835</t>
   </si>
   <si>
+    <t>1013383991</t>
+  </si>
+  <si>
+    <t>Alvarez Carlos Mario</t>
+  </si>
+  <si>
+    <t>Alvarez Arbelaez Hector Dario</t>
+  </si>
+  <si>
     <t>Alzate Villa William</t>
   </si>
   <si>
     <t>Castellanos Pinoz Johan Mateo</t>
   </si>
   <si>
+    <t>Arbelaez Londoño Alexander</t>
+  </si>
+  <si>
     <t>Arenas Villa Harold Alexander</t>
   </si>
   <si>
+    <t>Arias Jayer Juan David</t>
+  </si>
+  <si>
     <t>Artunduaga Cabrera Anderson</t>
   </si>
   <si>
+    <t>Atehortua Morales Didier</t>
+  </si>
+  <si>
+    <t>Y Esperanza - Cfe Iglesia Centro De Fe</t>
+  </si>
+  <si>
+    <t>Ortiz Monsalve Natalia</t>
+  </si>
+  <si>
+    <t>Blandon Tangarife Luis Fernando</t>
+  </si>
+  <si>
+    <t>Arrieta Mendoza Liseth</t>
+  </si>
+  <si>
+    <t>Buitrago Gonzalez Edison Alexander</t>
+  </si>
+  <si>
     <t>Mosquera Rodriguez Tania Karina</t>
   </si>
   <si>
+    <t>Cardona Villarreal Alba Mery</t>
+  </si>
+  <si>
+    <t>Castaño Zapata Jose Fernando</t>
+  </si>
+  <si>
+    <t>Viloria Montoya Isabel Cristina</t>
+  </si>
+  <si>
     <t>Chavarria Ramirez Roman Alberto</t>
   </si>
   <si>
+    <t>Chaverra Chaverra Juan David</t>
+  </si>
+  <si>
+    <t>Carreño Bohorquez Nora Maria</t>
+  </si>
+  <si>
+    <t>Correa Correa Mauricio</t>
+  </si>
+  <si>
+    <t>Correa Santana Edwin Andres</t>
+  </si>
+  <si>
     <t>Cortes Velasquez Juan Pablo</t>
   </si>
   <si>
     <t>Cuervo Paternina Eder Andres</t>
   </si>
   <si>
+    <t>De Luquez Diaz Ezequiel</t>
+  </si>
+  <si>
     <t>Diaz Rico John Edwin</t>
   </si>
   <si>
     <t>Echeverry Agudelo Sara Catalina</t>
   </si>
   <si>
-    <t>Ramirez Suarez Leidy Tatiana</t>
+    <t>Forero Reyes Janeth</t>
+  </si>
+  <si>
+    <t>Alvarez Cifuentes Jorge William</t>
+  </si>
+  <si>
+    <t>Correa Osorio Luisa Fernanda</t>
+  </si>
+  <si>
+    <t>Gonzalez Mora Julieth Marcela</t>
   </si>
   <si>
     <t>Garcia Valencia Cesar Augusto</t>
   </si>
   <si>
+    <t>Garzon Prieto Nelson Fidel</t>
+  </si>
+  <si>
+    <t>Cespedes Restrepo Maria Alejandra</t>
+  </si>
+  <si>
+    <t>Gil Clavijo Luber Mario</t>
+  </si>
+  <si>
+    <t>Avendaño Tamayo Yudi Patricia</t>
+  </si>
+  <si>
+    <t>Lozano Mosquera Mariam</t>
+  </si>
+  <si>
+    <t>Gomez Rios Geovanny Arley</t>
+  </si>
+  <si>
+    <t>Gonzalez Diaz Mauricio De Jesus</t>
+  </si>
+  <si>
+    <t>Gamboa Melendrez Jeniffer</t>
+  </si>
+  <si>
     <t>Ortiz Julio Sirly Dayana</t>
   </si>
   <si>
+    <t>Henao Betancur Jorge Humberto</t>
+  </si>
+  <si>
+    <t>Hurtado Orozco Yudi Andrea</t>
+  </si>
+  <si>
     <t>Agudelo Torres Sumilde Elena</t>
   </si>
   <si>
+    <t>Sanchez Isaura Pilar</t>
+  </si>
+  <si>
     <t>Rincon Lopera Liliana Maria</t>
   </si>
   <si>
     <t>Sas Inversiones Myt</t>
   </si>
   <si>
+    <t>Londoño Naranjo Zulma</t>
+  </si>
+  <si>
     <t>Manco Echavarria Reynel De Jesus</t>
   </si>
   <si>
     <t>Vergara Mejia Sara Valentina</t>
   </si>
   <si>
-    <t>Hernandez Morelo Liliana</t>
-  </si>
-  <si>
-    <t>Martinez Moreno Devinson</t>
+    <t>Mora Cardona Katherine</t>
   </si>
   <si>
     <t>Correa Mejia Catalina</t>
   </si>
   <si>
-    <t>Cardona Gaviria Maribel</t>
-  </si>
-  <si>
-    <t>Montoya Diaz Luis Fernando</t>
+    <t>Garcia Lancheros Yurani Yissel</t>
+  </si>
+  <si>
+    <t>Echeverri Gallego Monica Patricia</t>
   </si>
   <si>
     <t>Vellojin Cavadia Tania Marjolia</t>
   </si>
   <si>
+    <t>Orrego Zuluaga Juan Esteban</t>
+  </si>
+  <si>
     <t>Zabala Cuervo Diana Rocio</t>
   </si>
   <si>
     <t>Cano Guarin Sandra Milena</t>
   </si>
   <si>
+    <t>Ortiz Aristizabal Gabriel Jaime</t>
+  </si>
+  <si>
+    <t>Ospina Escobar Nilson James</t>
+  </si>
+  <si>
+    <t>Ospina Granda Diego Alexander</t>
+  </si>
+  <si>
+    <t>Ospina Diaz Carlos Arturo</t>
+  </si>
+  <si>
     <t>Perez Toro Juan Pablo</t>
   </si>
   <si>
+    <t>Peña Solórzano Francisco Javier</t>
+  </si>
+  <si>
+    <t>Pinzon Melchor Luis Ferney</t>
+  </si>
+  <si>
+    <t>Prieto Oyaga Cristhian Camilo</t>
+  </si>
+  <si>
+    <t>Puerta Mejia Luis Felipe</t>
+  </si>
+  <si>
     <t>Hernandez Cardona Mauricio</t>
   </si>
   <si>
     <t>Ramirez Urrutia Fredy</t>
   </si>
   <si>
+    <t>Callejas Acevedo Geovanny</t>
+  </si>
+  <si>
+    <t>Ramirez Ruiz Andres Julian</t>
+  </si>
+  <si>
+    <t>Restrepo Duque Jorge Mauricio</t>
+  </si>
+  <si>
     <t>Restrepo Silva Jeison</t>
   </si>
   <si>
     <t>Rizo Ibanez Jorge Armando</t>
   </si>
   <si>
+    <t>Marino Millan Yelitza Rossana</t>
+  </si>
+  <si>
+    <t>Rueda Piedrahita Carlos Ariel</t>
+  </si>
+  <si>
     <t>Agudelo Ruiz Sergio Mario</t>
   </si>
   <si>
@@ -556,6 +1030,12 @@
     <t>Sanchez Justiniano Martha Catherine</t>
   </si>
   <si>
+    <t>Sanchez Agudelo Uber Herney</t>
+  </si>
+  <si>
+    <t>Peña Morales Eliana Patricia</t>
+  </si>
+  <si>
     <t>Sayago Montes Juan Esteban</t>
   </si>
   <si>
@@ -568,7 +1048,13 @@
     <t>Arboleda Ramirez Daniel Andres</t>
   </si>
   <si>
-    <t>Hernandez Ospina Juan Camilo</t>
+    <t>Hernandez Baron Lina Paola</t>
+  </si>
+  <si>
+    <t>Suescun Gomez Jhony Alexander</t>
+  </si>
+  <si>
+    <t>Tabares Vergara Sergio Adrian</t>
   </si>
   <si>
     <t>Marin Osorio Johny Alexander</t>
@@ -577,24 +1063,45 @@
     <t>Troya Osorio Manuel Enrique</t>
   </si>
   <si>
+    <t>Usma Acevedo Elkin Humberto</t>
+  </si>
+  <si>
+    <t>Usuga Sepulveda Henrry</t>
+  </si>
+  <si>
     <t>Vanegas Zuñiga Ray Andres</t>
   </si>
   <si>
-    <t>Vasquez Gomez Alejandro</t>
+    <t>Vargas Ramos Ivan Isidro</t>
   </si>
   <si>
     <t>Ortiz Velez Laura Catalina</t>
   </si>
   <si>
+    <t>Villegas Gonzalez Wbeimar Alexander</t>
+  </si>
+  <si>
+    <t>Blanco Rincon Diana Margarita</t>
+  </si>
+  <si>
+    <t>Zapata Andrade Yicmar Lice</t>
+  </si>
+  <si>
     <t>Echeverry Giraldo Estefania</t>
   </si>
   <si>
+    <t>Zorrilla Adarve Oscar Wilfredo</t>
+  </si>
+  <si>
+    <t>QUINTO</t>
+  </si>
+  <si>
+    <t>DÉCIMO</t>
+  </si>
+  <si>
     <t>CUARTO</t>
   </si>
   <si>
-    <t>DÉCIMO</t>
-  </si>
-  <si>
     <t>ONCE</t>
   </si>
   <si>
@@ -604,9 +1111,6 @@
     <t>SEGUNDO</t>
   </si>
   <si>
-    <t>QUINTO</t>
-  </si>
-  <si>
     <t>TRANSICIÓN</t>
   </si>
   <si>
@@ -616,31 +1120,34 @@
     <t>SEXTO</t>
   </si>
   <si>
+    <t>NOVENO</t>
+  </si>
+  <si>
+    <t>PRIMERO</t>
+  </si>
+  <si>
     <t>TERCERO</t>
   </si>
   <si>
-    <t>NOVENO</t>
-  </si>
-  <si>
-    <t>PRIMERO</t>
-  </si>
-  <si>
-    <t>PRE-JARDIN</t>
-  </si>
-  <si>
-    <t>Junio - Julio</t>
-  </si>
-  <si>
-    <t>Abril - Mayo - Junio - Julio</t>
-  </si>
-  <si>
-    <t>Marzo - Abril - Mayo - Junio - Julio</t>
-  </si>
-  <si>
-    <t>Mayo - Junio - Julio</t>
-  </si>
-  <si>
-    <t>Febrero - Marzo - Abril - Mayo - Junio - Julio</t>
+    <t>Agosto</t>
+  </si>
+  <si>
+    <t>Julio - Agosto</t>
+  </si>
+  <si>
+    <t>Junio - Julio - Agosto</t>
+  </si>
+  <si>
+    <t>Abril - Mayo - Junio - Julio - Agosto</t>
+  </si>
+  <si>
+    <t>Mayo - Junio - Julio - Agosto</t>
+  </si>
+  <si>
+    <t>Febrero - Marzo - Abril - Mayo - Junio - Julio - Agosto</t>
+  </si>
+  <si>
+    <t>Marzo - Abril - Mayo - Junio - Julio - Agosto</t>
   </si>
 </sst>
 </file>
@@ -998,7 +1505,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M63"/>
+  <dimension ref="A1:M119"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:13">
@@ -1068,19 +1575,19 @@
         <v>19</v>
       </c>
       <c r="I2" t="s">
-        <v>81</v>
+        <v>137</v>
       </c>
       <c r="J2" t="s">
-        <v>143</v>
+        <v>255</v>
       </c>
       <c r="K2" t="s">
-        <v>191</v>
+        <v>359</v>
       </c>
       <c r="L2">
-        <v>1157256</v>
+        <v>577197</v>
       </c>
       <c r="M2" t="s">
-        <v>204</v>
+        <v>371</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -1109,19 +1616,19 @@
         <v>20</v>
       </c>
       <c r="I3" t="s">
-        <v>82</v>
+        <v>138</v>
       </c>
       <c r="J3" t="s">
-        <v>144</v>
+        <v>256</v>
       </c>
       <c r="K3" t="s">
-        <v>192</v>
+        <v>360</v>
       </c>
       <c r="L3">
-        <v>956502</v>
+        <v>414660</v>
       </c>
       <c r="M3" t="s">
-        <v>204</v>
+        <v>371</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -1150,19 +1657,19 @@
         <v>21</v>
       </c>
       <c r="I4" t="s">
-        <v>83</v>
+        <v>139</v>
       </c>
       <c r="J4" t="s">
-        <v>144</v>
+        <v>257</v>
       </c>
       <c r="K4" t="s">
-        <v>193</v>
+        <v>361</v>
       </c>
       <c r="L4">
-        <v>913296</v>
+        <v>1157132</v>
       </c>
       <c r="M4" t="s">
-        <v>204</v>
+        <v>372</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -1191,19 +1698,19 @@
         <v>22</v>
       </c>
       <c r="I5" t="s">
-        <v>84</v>
+        <v>140</v>
       </c>
       <c r="J5" t="s">
-        <v>145</v>
+        <v>258</v>
       </c>
       <c r="K5" t="s">
-        <v>194</v>
+        <v>360</v>
       </c>
       <c r="L5">
-        <v>2022880</v>
+        <v>477251</v>
       </c>
       <c r="M5" t="s">
-        <v>205</v>
+        <v>371</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -1232,19 +1739,19 @@
         <v>23</v>
       </c>
       <c r="I6" t="s">
-        <v>85</v>
+        <v>141</v>
       </c>
       <c r="J6" t="s">
-        <v>145</v>
+        <v>258</v>
       </c>
       <c r="K6" t="s">
-        <v>195</v>
+        <v>362</v>
       </c>
       <c r="L6">
-        <v>2537320</v>
+        <v>455648</v>
       </c>
       <c r="M6" t="s">
-        <v>205</v>
+        <v>371</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -1273,19 +1780,19 @@
         <v>24</v>
       </c>
       <c r="I7" t="s">
-        <v>86</v>
+        <v>142</v>
       </c>
       <c r="J7" t="s">
-        <v>146</v>
+        <v>259</v>
       </c>
       <c r="K7" t="s">
-        <v>196</v>
+        <v>361</v>
       </c>
       <c r="L7">
-        <v>1258720</v>
+        <v>626324</v>
       </c>
       <c r="M7" t="s">
-        <v>204</v>
+        <v>372</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -1314,19 +1821,19 @@
         <v>25</v>
       </c>
       <c r="I8" t="s">
-        <v>87</v>
+        <v>143</v>
       </c>
       <c r="J8" t="s">
-        <v>146</v>
+        <v>260</v>
       </c>
       <c r="K8" t="s">
-        <v>197</v>
+        <v>363</v>
       </c>
       <c r="L8">
-        <v>1229346</v>
+        <v>1033600</v>
       </c>
       <c r="M8" t="s">
-        <v>204</v>
+        <v>373</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -1355,19 +1862,19 @@
         <v>26</v>
       </c>
       <c r="I9" t="s">
-        <v>88</v>
+        <v>144</v>
       </c>
       <c r="J9" t="s">
-        <v>146</v>
+        <v>260</v>
       </c>
       <c r="K9" t="s">
-        <v>198</v>
+        <v>364</v>
       </c>
       <c r="L9">
-        <v>1198148</v>
+        <v>1676650</v>
       </c>
       <c r="M9" t="s">
-        <v>204</v>
+        <v>373</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -1396,19 +1903,19 @@
         <v>27</v>
       </c>
       <c r="I10" t="s">
-        <v>89</v>
+        <v>145</v>
       </c>
       <c r="J10" t="s">
-        <v>147</v>
+        <v>261</v>
       </c>
       <c r="K10" t="s">
-        <v>199</v>
+        <v>361</v>
       </c>
       <c r="L10">
-        <v>1242434</v>
+        <v>577876</v>
       </c>
       <c r="M10" t="s">
-        <v>204</v>
+        <v>371</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -1437,19 +1944,19 @@
         <v>28</v>
       </c>
       <c r="I11" t="s">
-        <v>90</v>
+        <v>146</v>
       </c>
       <c r="J11" t="s">
-        <v>147</v>
+        <v>262</v>
       </c>
       <c r="K11" t="s">
-        <v>195</v>
+        <v>359</v>
       </c>
       <c r="L11">
-        <v>2855968</v>
+        <v>628360</v>
       </c>
       <c r="M11" t="s">
-        <v>205</v>
+        <v>371</v>
       </c>
     </row>
     <row r="12" spans="1:13">
@@ -1478,19 +1985,19 @@
         <v>29</v>
       </c>
       <c r="I12" t="s">
-        <v>91</v>
+        <v>147</v>
       </c>
       <c r="J12" t="s">
-        <v>148</v>
+        <v>262</v>
       </c>
       <c r="K12" t="s">
-        <v>191</v>
+        <v>365</v>
       </c>
       <c r="L12">
-        <v>1080284</v>
+        <v>613673</v>
       </c>
       <c r="M12" t="s">
-        <v>204</v>
+        <v>371</v>
       </c>
     </row>
     <row r="13" spans="1:13">
@@ -1519,19 +2026,19 @@
         <v>30</v>
       </c>
       <c r="I13" t="s">
-        <v>92</v>
+        <v>148</v>
       </c>
       <c r="J13" t="s">
-        <v>149</v>
+        <v>263</v>
       </c>
       <c r="K13" t="s">
-        <v>194</v>
+        <v>359</v>
       </c>
       <c r="L13">
-        <v>2022880</v>
+        <v>557982</v>
       </c>
       <c r="M13" t="s">
-        <v>205</v>
+        <v>371</v>
       </c>
     </row>
     <row r="14" spans="1:13">
@@ -1560,19 +2067,19 @@
         <v>31</v>
       </c>
       <c r="I14" t="s">
-        <v>93</v>
+        <v>149</v>
       </c>
       <c r="J14" t="s">
-        <v>149</v>
+        <v>263</v>
       </c>
       <c r="K14" t="s">
-        <v>193</v>
+        <v>361</v>
       </c>
       <c r="L14">
-        <v>913296</v>
+        <v>577876</v>
       </c>
       <c r="M14" t="s">
-        <v>204</v>
+        <v>371</v>
       </c>
     </row>
     <row r="15" spans="1:13">
@@ -1601,19 +2108,19 @@
         <v>32</v>
       </c>
       <c r="I15" t="s">
-        <v>94</v>
+        <v>150</v>
       </c>
       <c r="J15" t="s">
-        <v>150</v>
+        <v>264</v>
       </c>
       <c r="K15" t="s">
-        <v>198</v>
+        <v>366</v>
       </c>
       <c r="L15">
-        <v>1265122</v>
+        <v>497612</v>
       </c>
       <c r="M15" t="s">
-        <v>204</v>
+        <v>371</v>
       </c>
     </row>
     <row r="16" spans="1:13">
@@ -1642,19 +2149,19 @@
         <v>33</v>
       </c>
       <c r="I16" t="s">
-        <v>95</v>
+        <v>151</v>
       </c>
       <c r="J16" t="s">
-        <v>151</v>
+        <v>265</v>
       </c>
       <c r="K16" t="s">
-        <v>192</v>
+        <v>359</v>
       </c>
       <c r="L16">
-        <v>956502</v>
+        <v>628360</v>
       </c>
       <c r="M16" t="s">
-        <v>204</v>
+        <v>371</v>
       </c>
     </row>
     <row r="17" spans="1:13">
@@ -1683,19 +2190,19 @@
         <v>34</v>
       </c>
       <c r="I17" t="s">
-        <v>96</v>
+        <v>152</v>
       </c>
       <c r="J17" t="s">
-        <v>152</v>
+        <v>266</v>
       </c>
       <c r="K17" t="s">
-        <v>192</v>
+        <v>359</v>
       </c>
       <c r="L17">
-        <v>1136976</v>
+        <v>593171</v>
       </c>
       <c r="M17" t="s">
-        <v>204</v>
+        <v>371</v>
       </c>
     </row>
     <row r="18" spans="1:13">
@@ -1724,19 +2231,19 @@
         <v>35</v>
       </c>
       <c r="I18" t="s">
-        <v>97</v>
+        <v>153</v>
       </c>
       <c r="J18" t="s">
-        <v>153</v>
+        <v>267</v>
       </c>
       <c r="K18" t="s">
-        <v>199</v>
+        <v>359</v>
       </c>
       <c r="L18">
-        <v>1917016</v>
+        <v>592197</v>
       </c>
       <c r="M18" t="s">
-        <v>205</v>
+        <v>371</v>
       </c>
     </row>
     <row r="19" spans="1:13">
@@ -1765,19 +2272,19 @@
         <v>36</v>
       </c>
       <c r="I19" t="s">
-        <v>98</v>
+        <v>154</v>
       </c>
       <c r="J19" t="s">
-        <v>154</v>
+        <v>268</v>
       </c>
       <c r="K19" t="s">
-        <v>200</v>
+        <v>359</v>
       </c>
       <c r="L19">
-        <v>2807794</v>
+        <v>405793</v>
       </c>
       <c r="M19" t="s">
-        <v>206</v>
+        <v>371</v>
       </c>
     </row>
     <row r="20" spans="1:13">
@@ -1806,19 +2313,19 @@
         <v>37</v>
       </c>
       <c r="I20" t="s">
-        <v>99</v>
+        <v>155</v>
       </c>
       <c r="J20" t="s">
-        <v>155</v>
+        <v>269</v>
       </c>
       <c r="K20" t="s">
-        <v>193</v>
+        <v>364</v>
       </c>
       <c r="L20">
-        <v>970440</v>
+        <v>2138976</v>
       </c>
       <c r="M20" t="s">
-        <v>204</v>
+        <v>373</v>
       </c>
     </row>
     <row r="21" spans="1:13">
@@ -1847,19 +2354,19 @@
         <v>38</v>
       </c>
       <c r="I21" t="s">
-        <v>100</v>
+        <v>156</v>
       </c>
       <c r="J21" t="s">
-        <v>155</v>
+        <v>270</v>
       </c>
       <c r="K21" t="s">
-        <v>200</v>
+        <v>359</v>
       </c>
       <c r="L21">
-        <v>1288964</v>
+        <v>357982</v>
       </c>
       <c r="M21" t="s">
-        <v>204</v>
+        <v>371</v>
       </c>
     </row>
     <row r="22" spans="1:13">
@@ -1888,19 +2395,19 @@
         <v>39</v>
       </c>
       <c r="I22" t="s">
-        <v>101</v>
+        <v>157</v>
       </c>
       <c r="J22" t="s">
-        <v>156</v>
+        <v>271</v>
       </c>
       <c r="K22" t="s">
-        <v>192</v>
+        <v>360</v>
       </c>
       <c r="L22">
-        <v>952506</v>
+        <v>892010</v>
       </c>
       <c r="M22" t="s">
-        <v>204</v>
+        <v>372</v>
       </c>
     </row>
     <row r="23" spans="1:13">
@@ -1929,19 +2436,19 @@
         <v>40</v>
       </c>
       <c r="I23" t="s">
-        <v>102</v>
+        <v>158</v>
       </c>
       <c r="J23" t="s">
-        <v>157</v>
+        <v>272</v>
       </c>
       <c r="K23" t="s">
-        <v>201</v>
+        <v>362</v>
       </c>
       <c r="L23">
-        <v>2710150</v>
+        <v>484054</v>
       </c>
       <c r="M23" t="s">
-        <v>206</v>
+        <v>371</v>
       </c>
     </row>
     <row r="24" spans="1:13">
@@ -1970,19 +2477,19 @@
         <v>41</v>
       </c>
       <c r="I24" t="s">
-        <v>103</v>
+        <v>159</v>
       </c>
       <c r="J24" t="s">
-        <v>158</v>
+        <v>273</v>
       </c>
       <c r="K24" t="s">
-        <v>201</v>
+        <v>361</v>
       </c>
       <c r="L24">
-        <v>1133616</v>
+        <v>1075712</v>
       </c>
       <c r="M24" t="s">
-        <v>204</v>
+        <v>372</v>
       </c>
     </row>
     <row r="25" spans="1:13">
@@ -2011,19 +2518,19 @@
         <v>42</v>
       </c>
       <c r="I25" t="s">
-        <v>104</v>
+        <v>160</v>
       </c>
       <c r="J25" t="s">
-        <v>159</v>
+        <v>274</v>
       </c>
       <c r="K25" t="s">
-        <v>192</v>
+        <v>361</v>
       </c>
       <c r="L25">
-        <v>955753</v>
+        <v>614324</v>
       </c>
       <c r="M25" t="s">
-        <v>204</v>
+        <v>371</v>
       </c>
     </row>
     <row r="26" spans="1:13">
@@ -2052,19 +2559,19 @@
         <v>43</v>
       </c>
       <c r="I26" t="s">
-        <v>105</v>
+        <v>161</v>
       </c>
       <c r="J26" t="s">
-        <v>160</v>
+        <v>275</v>
       </c>
       <c r="K26" t="s">
-        <v>202</v>
+        <v>367</v>
       </c>
       <c r="L26">
-        <v>1044902</v>
+        <v>1242434</v>
       </c>
       <c r="M26" t="s">
-        <v>204</v>
+        <v>372</v>
       </c>
     </row>
     <row r="27" spans="1:13">
@@ -2093,19 +2600,19 @@
         <v>44</v>
       </c>
       <c r="I27" t="s">
-        <v>106</v>
+        <v>162</v>
       </c>
       <c r="J27" t="s">
-        <v>161</v>
+        <v>276</v>
       </c>
       <c r="K27" t="s">
-        <v>198</v>
+        <v>360</v>
       </c>
       <c r="L27">
-        <v>1198148</v>
+        <v>506950</v>
       </c>
       <c r="M27" t="s">
-        <v>204</v>
+        <v>371</v>
       </c>
     </row>
     <row r="28" spans="1:13">
@@ -2134,19 +2641,19 @@
         <v>45</v>
       </c>
       <c r="I28" t="s">
-        <v>107</v>
+        <v>163</v>
       </c>
       <c r="J28" t="s">
-        <v>162</v>
+        <v>277</v>
       </c>
       <c r="K28" t="s">
-        <v>199</v>
+        <v>363</v>
       </c>
       <c r="L28">
-        <v>2353944</v>
+        <v>502720</v>
       </c>
       <c r="M28" t="s">
-        <v>205</v>
+        <v>371</v>
       </c>
     </row>
     <row r="29" spans="1:13">
@@ -2175,19 +2682,19 @@
         <v>46</v>
       </c>
       <c r="I29" t="s">
-        <v>108</v>
+        <v>164</v>
       </c>
       <c r="J29" t="s">
-        <v>163</v>
+        <v>278</v>
       </c>
       <c r="K29" t="s">
-        <v>193</v>
+        <v>363</v>
       </c>
       <c r="L29">
-        <v>969160</v>
+        <v>2533600</v>
       </c>
       <c r="M29" t="s">
-        <v>204</v>
+        <v>374</v>
       </c>
     </row>
     <row r="30" spans="1:13">
@@ -2216,19 +2723,19 @@
         <v>47</v>
       </c>
       <c r="I30" t="s">
-        <v>109</v>
+        <v>165</v>
       </c>
       <c r="J30" t="s">
-        <v>164</v>
+        <v>278</v>
       </c>
       <c r="K30" t="s">
-        <v>199</v>
+        <v>362</v>
       </c>
       <c r="L30">
-        <v>1651524</v>
+        <v>1372944</v>
       </c>
       <c r="M30" t="s">
-        <v>207</v>
+        <v>373</v>
       </c>
     </row>
     <row r="31" spans="1:13">
@@ -2257,19 +2764,19 @@
         <v>48</v>
       </c>
       <c r="I31" t="s">
-        <v>110</v>
+        <v>166</v>
       </c>
       <c r="J31" t="s">
-        <v>165</v>
+        <v>279</v>
       </c>
       <c r="K31" t="s">
-        <v>203</v>
+        <v>366</v>
       </c>
       <c r="L31">
-        <v>1416696</v>
+        <v>631561</v>
       </c>
       <c r="M31" t="s">
-        <v>204</v>
+        <v>371</v>
       </c>
     </row>
     <row r="32" spans="1:13">
@@ -2298,19 +2805,19 @@
         <v>49</v>
       </c>
       <c r="I32" t="s">
-        <v>111</v>
+        <v>167</v>
       </c>
       <c r="J32" t="s">
-        <v>165</v>
+        <v>280</v>
       </c>
       <c r="K32" t="s">
-        <v>197</v>
+        <v>360</v>
       </c>
       <c r="L32">
-        <v>1160620</v>
+        <v>567488</v>
       </c>
       <c r="M32" t="s">
-        <v>204</v>
+        <v>371</v>
       </c>
     </row>
     <row r="33" spans="1:13">
@@ -2339,19 +2846,19 @@
         <v>50</v>
       </c>
       <c r="I33" t="s">
-        <v>112</v>
+        <v>168</v>
       </c>
       <c r="J33" t="s">
-        <v>165</v>
+        <v>281</v>
       </c>
       <c r="K33" t="s">
-        <v>195</v>
+        <v>360</v>
       </c>
       <c r="L33">
-        <v>1344322</v>
+        <v>1437753</v>
       </c>
       <c r="M33" t="s">
-        <v>204</v>
+        <v>373</v>
       </c>
     </row>
     <row r="34" spans="1:13">
@@ -2380,19 +2887,19 @@
         <v>51</v>
       </c>
       <c r="I34" t="s">
-        <v>113</v>
+        <v>169</v>
       </c>
       <c r="J34" t="s">
-        <v>166</v>
+        <v>282</v>
       </c>
       <c r="K34" t="s">
-        <v>192</v>
+        <v>360</v>
       </c>
       <c r="L34">
-        <v>3073980</v>
+        <v>1708464</v>
       </c>
       <c r="M34" t="s">
-        <v>208</v>
+        <v>373</v>
       </c>
     </row>
     <row r="35" spans="1:13">
@@ -2421,19 +2928,19 @@
         <v>52</v>
       </c>
       <c r="I35" t="s">
-        <v>114</v>
+        <v>170</v>
       </c>
       <c r="J35" t="s">
-        <v>167</v>
+        <v>283</v>
       </c>
       <c r="K35" t="s">
-        <v>191</v>
+        <v>368</v>
       </c>
       <c r="L35">
-        <v>815648</v>
+        <v>1078060</v>
       </c>
       <c r="M35" t="s">
-        <v>204</v>
+        <v>372</v>
       </c>
     </row>
     <row r="36" spans="1:13">
@@ -2462,19 +2969,19 @@
         <v>53</v>
       </c>
       <c r="I36" t="s">
-        <v>115</v>
+        <v>171</v>
       </c>
       <c r="J36" t="s">
-        <v>168</v>
+        <v>284</v>
       </c>
       <c r="K36" t="s">
-        <v>202</v>
+        <v>369</v>
       </c>
       <c r="L36">
-        <v>1190353</v>
+        <v>488574</v>
       </c>
       <c r="M36" t="s">
-        <v>207</v>
+        <v>371</v>
       </c>
     </row>
     <row r="37" spans="1:13">
@@ -2503,19 +3010,19 @@
         <v>54</v>
       </c>
       <c r="I37" t="s">
-        <v>116</v>
+        <v>172</v>
       </c>
       <c r="J37" t="s">
-        <v>169</v>
+        <v>285</v>
       </c>
       <c r="K37" t="s">
-        <v>191</v>
+        <v>363</v>
       </c>
       <c r="L37">
-        <v>1224620</v>
+        <v>1007440</v>
       </c>
       <c r="M37" t="s">
-        <v>204</v>
+        <v>372</v>
       </c>
     </row>
     <row r="38" spans="1:13">
@@ -2544,19 +3051,19 @@
         <v>55</v>
       </c>
       <c r="I38" t="s">
-        <v>117</v>
+        <v>173</v>
       </c>
       <c r="J38" t="s">
-        <v>170</v>
+        <v>286</v>
       </c>
       <c r="K38" t="s">
-        <v>194</v>
+        <v>368</v>
       </c>
       <c r="L38">
-        <v>2941320</v>
+        <v>538030</v>
       </c>
       <c r="M38" t="s">
-        <v>208</v>
+        <v>371</v>
       </c>
     </row>
     <row r="39" spans="1:13">
@@ -2585,19 +3092,19 @@
         <v>56</v>
       </c>
       <c r="I39" t="s">
-        <v>118</v>
+        <v>174</v>
       </c>
       <c r="J39" t="s">
-        <v>171</v>
+        <v>287</v>
       </c>
       <c r="K39" t="s">
-        <v>192</v>
+        <v>370</v>
       </c>
       <c r="L39">
-        <v>914782</v>
+        <v>2419093</v>
       </c>
       <c r="M39" t="s">
-        <v>204</v>
+        <v>375</v>
       </c>
     </row>
     <row r="40" spans="1:13">
@@ -2626,19 +3133,19 @@
         <v>57</v>
       </c>
       <c r="I40" t="s">
-        <v>119</v>
+        <v>175</v>
       </c>
       <c r="J40" t="s">
-        <v>171</v>
+        <v>288</v>
       </c>
       <c r="K40" t="s">
-        <v>198</v>
+        <v>368</v>
       </c>
       <c r="L40">
-        <v>1015962</v>
+        <v>1014246</v>
       </c>
       <c r="M40" t="s">
-        <v>204</v>
+        <v>372</v>
       </c>
     </row>
     <row r="41" spans="1:13">
@@ -2667,19 +3174,19 @@
         <v>58</v>
       </c>
       <c r="I41" t="s">
-        <v>120</v>
+        <v>176</v>
       </c>
       <c r="J41" t="s">
-        <v>172</v>
+        <v>289</v>
       </c>
       <c r="K41" t="s">
-        <v>200</v>
+        <v>368</v>
       </c>
       <c r="L41">
-        <v>1241196</v>
+        <v>500292</v>
       </c>
       <c r="M41" t="s">
-        <v>207</v>
+        <v>371</v>
       </c>
     </row>
     <row r="42" spans="1:13">
@@ -2708,19 +3215,19 @@
         <v>59</v>
       </c>
       <c r="I42" t="s">
-        <v>121</v>
+        <v>177</v>
       </c>
       <c r="J42" t="s">
-        <v>172</v>
+        <v>289</v>
       </c>
       <c r="K42" t="s">
-        <v>194</v>
+        <v>364</v>
       </c>
       <c r="L42">
-        <v>1513600</v>
+        <v>601960</v>
       </c>
       <c r="M42" t="s">
-        <v>207</v>
+        <v>371</v>
       </c>
     </row>
     <row r="43" spans="1:13">
@@ -2749,19 +3256,19 @@
         <v>60</v>
       </c>
       <c r="I43" t="s">
-        <v>122</v>
+        <v>178</v>
       </c>
       <c r="J43" t="s">
-        <v>173</v>
+        <v>290</v>
       </c>
       <c r="K43" t="s">
-        <v>196</v>
+        <v>359</v>
       </c>
       <c r="L43">
-        <v>1258720</v>
+        <v>593171</v>
       </c>
       <c r="M43" t="s">
-        <v>204</v>
+        <v>371</v>
       </c>
     </row>
     <row r="44" spans="1:13">
@@ -2790,19 +3297,19 @@
         <v>61</v>
       </c>
       <c r="I44" t="s">
-        <v>123</v>
+        <v>179</v>
       </c>
       <c r="J44" t="s">
-        <v>173</v>
+        <v>291</v>
       </c>
       <c r="K44" t="s">
-        <v>202</v>
+        <v>361</v>
       </c>
       <c r="L44">
-        <v>1176410</v>
+        <v>540996</v>
       </c>
       <c r="M44" t="s">
-        <v>204</v>
+        <v>371</v>
       </c>
     </row>
     <row r="45" spans="1:13">
@@ -2831,19 +3338,19 @@
         <v>62</v>
       </c>
       <c r="I45" t="s">
-        <v>124</v>
+        <v>180</v>
       </c>
       <c r="J45" t="s">
-        <v>174</v>
+        <v>292</v>
       </c>
       <c r="K45" t="s">
-        <v>192</v>
+        <v>359</v>
       </c>
       <c r="L45">
-        <v>955506</v>
+        <v>1258720</v>
       </c>
       <c r="M45" t="s">
-        <v>204</v>
+        <v>372</v>
       </c>
     </row>
     <row r="46" spans="1:13">
@@ -2872,19 +3379,19 @@
         <v>63</v>
       </c>
       <c r="I46" t="s">
-        <v>125</v>
+        <v>181</v>
       </c>
       <c r="J46" t="s">
-        <v>175</v>
+        <v>293</v>
       </c>
       <c r="K46" t="s">
-        <v>193</v>
+        <v>362</v>
       </c>
       <c r="L46">
-        <v>968160</v>
+        <v>970720</v>
       </c>
       <c r="M46" t="s">
-        <v>204</v>
+        <v>372</v>
       </c>
     </row>
     <row r="47" spans="1:13">
@@ -2913,19 +3420,19 @@
         <v>64</v>
       </c>
       <c r="I47" t="s">
-        <v>126</v>
+        <v>182</v>
       </c>
       <c r="J47" t="s">
-        <v>176</v>
+        <v>294</v>
       </c>
       <c r="K47" t="s">
-        <v>193</v>
+        <v>363</v>
       </c>
       <c r="L47">
-        <v>970660</v>
+        <v>396871</v>
       </c>
       <c r="M47" t="s">
-        <v>204</v>
+        <v>371</v>
       </c>
     </row>
     <row r="48" spans="1:13">
@@ -2954,19 +3461,19 @@
         <v>65</v>
       </c>
       <c r="I48" t="s">
-        <v>127</v>
+        <v>183</v>
       </c>
       <c r="J48" t="s">
-        <v>177</v>
+        <v>294</v>
       </c>
       <c r="K48" t="s">
-        <v>191</v>
+        <v>360</v>
       </c>
       <c r="L48">
-        <v>1773944</v>
+        <v>376786</v>
       </c>
       <c r="M48" t="s">
-        <v>207</v>
+        <v>371</v>
       </c>
     </row>
     <row r="49" spans="1:13">
@@ -2995,19 +3502,19 @@
         <v>66</v>
       </c>
       <c r="I49" t="s">
-        <v>128</v>
+        <v>184</v>
       </c>
       <c r="J49" t="s">
-        <v>178</v>
+        <v>295</v>
       </c>
       <c r="K49" t="s">
-        <v>201</v>
+        <v>359</v>
       </c>
       <c r="L49">
-        <v>1524369</v>
+        <v>557982</v>
       </c>
       <c r="M49" t="s">
-        <v>207</v>
+        <v>371</v>
       </c>
     </row>
     <row r="50" spans="1:13">
@@ -3036,19 +3543,19 @@
         <v>67</v>
       </c>
       <c r="I50" t="s">
-        <v>129</v>
+        <v>185</v>
       </c>
       <c r="J50" t="s">
-        <v>178</v>
+        <v>296</v>
       </c>
       <c r="K50" t="s">
-        <v>193</v>
+        <v>362</v>
       </c>
       <c r="L50">
-        <v>913296</v>
+        <v>178800</v>
       </c>
       <c r="M50" t="s">
-        <v>204</v>
+        <v>371</v>
       </c>
     </row>
     <row r="51" spans="1:13">
@@ -3077,19 +3584,19 @@
         <v>68</v>
       </c>
       <c r="I51" t="s">
-        <v>130</v>
+        <v>186</v>
       </c>
       <c r="J51" t="s">
-        <v>178</v>
+        <v>297</v>
       </c>
       <c r="K51" t="s">
-        <v>199</v>
+        <v>370</v>
       </c>
       <c r="L51">
-        <v>1658262</v>
+        <v>602093</v>
       </c>
       <c r="M51" t="s">
-        <v>207</v>
+        <v>371</v>
       </c>
     </row>
     <row r="52" spans="1:13">
@@ -3118,19 +3625,19 @@
         <v>69</v>
       </c>
       <c r="I52" t="s">
-        <v>131</v>
+        <v>187</v>
       </c>
       <c r="J52" t="s">
-        <v>179</v>
+        <v>298</v>
       </c>
       <c r="K52" t="s">
-        <v>200</v>
+        <v>359</v>
       </c>
       <c r="L52">
-        <v>2657794</v>
+        <v>519793</v>
       </c>
       <c r="M52" t="s">
-        <v>206</v>
+        <v>371</v>
       </c>
     </row>
     <row r="53" spans="1:13">
@@ -3159,19 +3666,19 @@
         <v>70</v>
       </c>
       <c r="I53" t="s">
-        <v>132</v>
+        <v>188</v>
       </c>
       <c r="J53" t="s">
-        <v>180</v>
+        <v>299</v>
       </c>
       <c r="K53" t="s">
-        <v>195</v>
+        <v>360</v>
       </c>
       <c r="L53">
-        <v>4295952</v>
+        <v>439757</v>
       </c>
       <c r="M53" t="s">
-        <v>208</v>
+        <v>371</v>
       </c>
     </row>
     <row r="54" spans="1:13">
@@ -3200,19 +3707,19 @@
         <v>71</v>
       </c>
       <c r="I54" t="s">
-        <v>133</v>
+        <v>189</v>
       </c>
       <c r="J54" t="s">
-        <v>181</v>
+        <v>300</v>
       </c>
       <c r="K54" t="s">
-        <v>194</v>
+        <v>363</v>
       </c>
       <c r="L54">
-        <v>2276408</v>
+        <v>1070822</v>
       </c>
       <c r="M54" t="s">
-        <v>205</v>
+        <v>372</v>
       </c>
     </row>
     <row r="55" spans="1:13">
@@ -3241,19 +3748,19 @@
         <v>72</v>
       </c>
       <c r="I55" t="s">
-        <v>134</v>
+        <v>190</v>
       </c>
       <c r="J55" t="s">
-        <v>182</v>
+        <v>301</v>
       </c>
       <c r="K55" t="s">
-        <v>192</v>
+        <v>368</v>
       </c>
       <c r="L55">
-        <v>1527990</v>
+        <v>2164120</v>
       </c>
       <c r="M55" t="s">
-        <v>207</v>
+        <v>375</v>
       </c>
     </row>
     <row r="56" spans="1:13">
@@ -3282,19 +3789,19 @@
         <v>73</v>
       </c>
       <c r="I56" t="s">
-        <v>135</v>
+        <v>191</v>
       </c>
       <c r="J56" t="s">
-        <v>183</v>
+        <v>302</v>
       </c>
       <c r="K56" t="s">
-        <v>192</v>
+        <v>368</v>
       </c>
       <c r="L56">
-        <v>956502</v>
+        <v>1707552</v>
       </c>
       <c r="M56" t="s">
-        <v>204</v>
+        <v>373</v>
       </c>
     </row>
     <row r="57" spans="1:13">
@@ -3323,19 +3830,19 @@
         <v>74</v>
       </c>
       <c r="I57" t="s">
-        <v>136</v>
+        <v>192</v>
       </c>
       <c r="J57" t="s">
-        <v>184</v>
+        <v>303</v>
       </c>
       <c r="K57" t="s">
-        <v>194</v>
+        <v>359</v>
       </c>
       <c r="L57">
-        <v>1791600</v>
+        <v>593171</v>
       </c>
       <c r="M57" t="s">
-        <v>205</v>
+        <v>371</v>
       </c>
     </row>
     <row r="58" spans="1:13">
@@ -3364,19 +3871,19 @@
         <v>75</v>
       </c>
       <c r="I58" t="s">
-        <v>137</v>
+        <v>193</v>
       </c>
       <c r="J58" t="s">
-        <v>185</v>
+        <v>304</v>
       </c>
       <c r="K58" t="s">
-        <v>196</v>
+        <v>360</v>
       </c>
       <c r="L58">
-        <v>1182855</v>
+        <v>477251</v>
       </c>
       <c r="M58" t="s">
-        <v>204</v>
+        <v>371</v>
       </c>
     </row>
     <row r="59" spans="1:13">
@@ -3405,19 +3912,19 @@
         <v>76</v>
       </c>
       <c r="I59" t="s">
-        <v>138</v>
+        <v>194</v>
       </c>
       <c r="J59" t="s">
-        <v>186</v>
+        <v>305</v>
       </c>
       <c r="K59" t="s">
-        <v>194</v>
+        <v>369</v>
       </c>
       <c r="L59">
-        <v>2812103</v>
+        <v>521451</v>
       </c>
       <c r="M59" t="s">
-        <v>208</v>
+        <v>371</v>
       </c>
     </row>
     <row r="60" spans="1:13">
@@ -3446,19 +3953,19 @@
         <v>77</v>
       </c>
       <c r="I60" t="s">
-        <v>139</v>
+        <v>195</v>
       </c>
       <c r="J60" t="s">
-        <v>187</v>
+        <v>306</v>
       </c>
       <c r="K60" t="s">
-        <v>196</v>
+        <v>364</v>
       </c>
       <c r="L60">
-        <v>1047586</v>
+        <v>176330</v>
       </c>
       <c r="M60" t="s">
-        <v>204</v>
+        <v>371</v>
       </c>
     </row>
     <row r="61" spans="1:13">
@@ -3487,19 +3994,19 @@
         <v>78</v>
       </c>
       <c r="I61" t="s">
-        <v>140</v>
+        <v>196</v>
       </c>
       <c r="J61" t="s">
-        <v>188</v>
+        <v>307</v>
       </c>
       <c r="K61" t="s">
-        <v>199</v>
+        <v>362</v>
       </c>
       <c r="L61">
-        <v>1762458</v>
+        <v>1457520</v>
       </c>
       <c r="M61" t="s">
-        <v>207</v>
+        <v>373</v>
       </c>
     </row>
     <row r="62" spans="1:13">
@@ -3528,19 +4035,19 @@
         <v>79</v>
       </c>
       <c r="I62" t="s">
-        <v>141</v>
+        <v>197</v>
       </c>
       <c r="J62" t="s">
-        <v>189</v>
+        <v>308</v>
       </c>
       <c r="K62" t="s">
-        <v>199</v>
+        <v>361</v>
       </c>
       <c r="L62">
-        <v>3126138</v>
+        <v>1133690</v>
       </c>
       <c r="M62" t="s">
-        <v>208</v>
+        <v>372</v>
       </c>
     </row>
     <row r="63" spans="1:13">
@@ -3569,19 +4076,2315 @@
         <v>80</v>
       </c>
       <c r="I63" t="s">
-        <v>142</v>
+        <v>198</v>
       </c>
       <c r="J63" t="s">
-        <v>190</v>
+        <v>309</v>
       </c>
       <c r="K63" t="s">
-        <v>195</v>
+        <v>360</v>
       </c>
       <c r="L63">
-        <v>1343966</v>
+        <v>507330</v>
       </c>
       <c r="M63" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="64" spans="1:13">
+      <c r="A64" t="s">
+        <v>13</v>
+      </c>
+      <c r="B64" t="s">
+        <v>14</v>
+      </c>
+      <c r="C64">
+        <v>2026</v>
+      </c>
+      <c r="D64" t="s">
+        <v>15</v>
+      </c>
+      <c r="E64" t="s">
+        <v>16</v>
+      </c>
+      <c r="F64" t="s">
+        <v>17</v>
+      </c>
+      <c r="G64" t="s">
+        <v>18</v>
+      </c>
+      <c r="H64" t="s">
+        <v>81</v>
+      </c>
+      <c r="I64" t="s">
+        <v>199</v>
+      </c>
+      <c r="J64" t="s">
+        <v>310</v>
+      </c>
+      <c r="K64" t="s">
+        <v>360</v>
+      </c>
+      <c r="L64">
+        <v>3593310</v>
+      </c>
+      <c r="M64" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="65" spans="1:13">
+      <c r="A65" t="s">
+        <v>13</v>
+      </c>
+      <c r="B65" t="s">
+        <v>14</v>
+      </c>
+      <c r="C65">
+        <v>2026</v>
+      </c>
+      <c r="D65" t="s">
+        <v>15</v>
+      </c>
+      <c r="E65" t="s">
+        <v>16</v>
+      </c>
+      <c r="F65" t="s">
+        <v>17</v>
+      </c>
+      <c r="G65" t="s">
+        <v>18</v>
+      </c>
+      <c r="H65" t="s">
+        <v>82</v>
+      </c>
+      <c r="I65" t="s">
+        <v>200</v>
+      </c>
+      <c r="J65" t="s">
+        <v>311</v>
+      </c>
+      <c r="K65" t="s">
+        <v>370</v>
+      </c>
+      <c r="L65">
+        <v>1441698</v>
+      </c>
+      <c r="M65" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="66" spans="1:13">
+      <c r="A66" t="s">
+        <v>13</v>
+      </c>
+      <c r="B66" t="s">
+        <v>14</v>
+      </c>
+      <c r="C66">
+        <v>2026</v>
+      </c>
+      <c r="D66" t="s">
+        <v>15</v>
+      </c>
+      <c r="E66" t="s">
+        <v>16</v>
+      </c>
+      <c r="F66" t="s">
+        <v>17</v>
+      </c>
+      <c r="G66" t="s">
+        <v>18</v>
+      </c>
+      <c r="H66" t="s">
+        <v>83</v>
+      </c>
+      <c r="I66" t="s">
+        <v>201</v>
+      </c>
+      <c r="J66" t="s">
+        <v>312</v>
+      </c>
+      <c r="K66" t="s">
+        <v>361</v>
+      </c>
+      <c r="L66">
+        <v>568972</v>
+      </c>
+      <c r="M66" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="67" spans="1:13">
+      <c r="A67" t="s">
+        <v>13</v>
+      </c>
+      <c r="B67" t="s">
+        <v>14</v>
+      </c>
+      <c r="C67">
+        <v>2026</v>
+      </c>
+      <c r="D67" t="s">
+        <v>15</v>
+      </c>
+      <c r="E67" t="s">
+        <v>16</v>
+      </c>
+      <c r="F67" t="s">
+        <v>17</v>
+      </c>
+      <c r="G67" t="s">
+        <v>18</v>
+      </c>
+      <c r="H67" t="s">
+        <v>84</v>
+      </c>
+      <c r="I67" t="s">
+        <v>202</v>
+      </c>
+      <c r="J67" t="s">
+        <v>313</v>
+      </c>
+      <c r="K67" t="s">
+        <v>369</v>
+      </c>
+      <c r="L67">
+        <v>1044902</v>
+      </c>
+      <c r="M67" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="68" spans="1:13">
+      <c r="A68" t="s">
+        <v>13</v>
+      </c>
+      <c r="B68" t="s">
+        <v>14</v>
+      </c>
+      <c r="C68">
+        <v>2026</v>
+      </c>
+      <c r="D68" t="s">
+        <v>15</v>
+      </c>
+      <c r="E68" t="s">
+        <v>16</v>
+      </c>
+      <c r="F68" t="s">
+        <v>17</v>
+      </c>
+      <c r="G68" t="s">
+        <v>18</v>
+      </c>
+      <c r="H68" t="s">
+        <v>85</v>
+      </c>
+      <c r="I68" t="s">
+        <v>203</v>
+      </c>
+      <c r="J68" t="s">
+        <v>314</v>
+      </c>
+      <c r="K68" t="s">
+        <v>362</v>
+      </c>
+      <c r="L68">
+        <v>517072</v>
+      </c>
+      <c r="M68" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="69" spans="1:13">
+      <c r="A69" t="s">
+        <v>13</v>
+      </c>
+      <c r="B69" t="s">
+        <v>14</v>
+      </c>
+      <c r="C69">
+        <v>2026</v>
+      </c>
+      <c r="D69" t="s">
+        <v>15</v>
+      </c>
+      <c r="E69" t="s">
+        <v>16</v>
+      </c>
+      <c r="F69" t="s">
+        <v>17</v>
+      </c>
+      <c r="G69" t="s">
+        <v>18</v>
+      </c>
+      <c r="H69" t="s">
+        <v>86</v>
+      </c>
+      <c r="I69" t="s">
         <v>204</v>
+      </c>
+      <c r="J69" t="s">
+        <v>315</v>
+      </c>
+      <c r="K69" t="s">
+        <v>361</v>
+      </c>
+      <c r="L69">
+        <v>577876</v>
+      </c>
+      <c r="M69" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="70" spans="1:13">
+      <c r="A70" t="s">
+        <v>13</v>
+      </c>
+      <c r="B70" t="s">
+        <v>14</v>
+      </c>
+      <c r="C70">
+        <v>2026</v>
+      </c>
+      <c r="D70" t="s">
+        <v>15</v>
+      </c>
+      <c r="E70" t="s">
+        <v>16</v>
+      </c>
+      <c r="F70" t="s">
+        <v>17</v>
+      </c>
+      <c r="G70" t="s">
+        <v>18</v>
+      </c>
+      <c r="H70" t="s">
+        <v>87</v>
+      </c>
+      <c r="I70" t="s">
+        <v>205</v>
+      </c>
+      <c r="J70" t="s">
+        <v>316</v>
+      </c>
+      <c r="K70" t="s">
+        <v>368</v>
+      </c>
+      <c r="L70">
+        <v>601684</v>
+      </c>
+      <c r="M70" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="71" spans="1:13">
+      <c r="A71" t="s">
+        <v>13</v>
+      </c>
+      <c r="B71" t="s">
+        <v>14</v>
+      </c>
+      <c r="C71">
+        <v>2026</v>
+      </c>
+      <c r="D71" t="s">
+        <v>15</v>
+      </c>
+      <c r="E71" t="s">
+        <v>16</v>
+      </c>
+      <c r="F71" t="s">
+        <v>17</v>
+      </c>
+      <c r="G71" t="s">
+        <v>18</v>
+      </c>
+      <c r="H71" t="s">
+        <v>88</v>
+      </c>
+      <c r="I71" t="s">
+        <v>206</v>
+      </c>
+      <c r="J71" t="s">
+        <v>317</v>
+      </c>
+      <c r="K71" t="s">
+        <v>362</v>
+      </c>
+      <c r="L71">
+        <v>438520</v>
+      </c>
+      <c r="M71" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="72" spans="1:13">
+      <c r="A72" t="s">
+        <v>13</v>
+      </c>
+      <c r="B72" t="s">
+        <v>14</v>
+      </c>
+      <c r="C72">
+        <v>2026</v>
+      </c>
+      <c r="D72" t="s">
+        <v>15</v>
+      </c>
+      <c r="E72" t="s">
+        <v>16</v>
+      </c>
+      <c r="F72" t="s">
+        <v>17</v>
+      </c>
+      <c r="G72" t="s">
+        <v>18</v>
+      </c>
+      <c r="H72" t="s">
+        <v>89</v>
+      </c>
+      <c r="I72" t="s">
+        <v>207</v>
+      </c>
+      <c r="J72" t="s">
+        <v>318</v>
+      </c>
+      <c r="K72" t="s">
+        <v>361</v>
+      </c>
+      <c r="L72">
+        <v>1230648</v>
+      </c>
+      <c r="M72" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="73" spans="1:13">
+      <c r="A73" t="s">
+        <v>13</v>
+      </c>
+      <c r="B73" t="s">
+        <v>14</v>
+      </c>
+      <c r="C73">
+        <v>2026</v>
+      </c>
+      <c r="D73" t="s">
+        <v>15</v>
+      </c>
+      <c r="E73" t="s">
+        <v>16</v>
+      </c>
+      <c r="F73" t="s">
+        <v>17</v>
+      </c>
+      <c r="G73" t="s">
+        <v>18</v>
+      </c>
+      <c r="H73" t="s">
+        <v>90</v>
+      </c>
+      <c r="I73" t="s">
+        <v>208</v>
+      </c>
+      <c r="J73" t="s">
+        <v>319</v>
+      </c>
+      <c r="K73" t="s">
+        <v>359</v>
+      </c>
+      <c r="L73">
+        <v>579197</v>
+      </c>
+      <c r="M73" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="74" spans="1:13">
+      <c r="A74" t="s">
+        <v>13</v>
+      </c>
+      <c r="B74" t="s">
+        <v>14</v>
+      </c>
+      <c r="C74">
+        <v>2026</v>
+      </c>
+      <c r="D74" t="s">
+        <v>15</v>
+      </c>
+      <c r="E74" t="s">
+        <v>16</v>
+      </c>
+      <c r="F74" t="s">
+        <v>17</v>
+      </c>
+      <c r="G74" t="s">
+        <v>18</v>
+      </c>
+      <c r="H74" t="s">
+        <v>91</v>
+      </c>
+      <c r="I74" t="s">
+        <v>209</v>
+      </c>
+      <c r="J74" t="s">
+        <v>320</v>
+      </c>
+      <c r="K74" t="s">
+        <v>359</v>
+      </c>
+      <c r="L74">
+        <v>628360</v>
+      </c>
+      <c r="M74" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="75" spans="1:13">
+      <c r="A75" t="s">
+        <v>13</v>
+      </c>
+      <c r="B75" t="s">
+        <v>14</v>
+      </c>
+      <c r="C75">
+        <v>2026</v>
+      </c>
+      <c r="D75" t="s">
+        <v>15</v>
+      </c>
+      <c r="E75" t="s">
+        <v>16</v>
+      </c>
+      <c r="F75" t="s">
+        <v>17</v>
+      </c>
+      <c r="G75" t="s">
+        <v>18</v>
+      </c>
+      <c r="H75" t="s">
+        <v>92</v>
+      </c>
+      <c r="I75" t="s">
+        <v>210</v>
+      </c>
+      <c r="J75" t="s">
+        <v>321</v>
+      </c>
+      <c r="K75" t="s">
+        <v>370</v>
+      </c>
+      <c r="L75">
+        <v>1212598</v>
+      </c>
+      <c r="M75" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="76" spans="1:13">
+      <c r="A76" t="s">
+        <v>13</v>
+      </c>
+      <c r="B76" t="s">
+        <v>14</v>
+      </c>
+      <c r="C76">
+        <v>2026</v>
+      </c>
+      <c r="D76" t="s">
+        <v>15</v>
+      </c>
+      <c r="E76" t="s">
+        <v>16</v>
+      </c>
+      <c r="F76" t="s">
+        <v>17</v>
+      </c>
+      <c r="G76" t="s">
+        <v>18</v>
+      </c>
+      <c r="H76" t="s">
+        <v>93</v>
+      </c>
+      <c r="I76" t="s">
+        <v>211</v>
+      </c>
+      <c r="J76" t="s">
+        <v>322</v>
+      </c>
+      <c r="K76" t="s">
+        <v>363</v>
+      </c>
+      <c r="L76">
+        <v>481170</v>
+      </c>
+      <c r="M76" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="77" spans="1:13">
+      <c r="A77" t="s">
+        <v>13</v>
+      </c>
+      <c r="B77" t="s">
+        <v>14</v>
+      </c>
+      <c r="C77">
+        <v>2026</v>
+      </c>
+      <c r="D77" t="s">
+        <v>15</v>
+      </c>
+      <c r="E77" t="s">
+        <v>16</v>
+      </c>
+      <c r="F77" t="s">
+        <v>17</v>
+      </c>
+      <c r="G77" t="s">
+        <v>18</v>
+      </c>
+      <c r="H77" t="s">
+        <v>94</v>
+      </c>
+      <c r="I77" t="s">
+        <v>212</v>
+      </c>
+      <c r="J77" t="s">
+        <v>323</v>
+      </c>
+      <c r="K77" t="s">
+        <v>363</v>
+      </c>
+      <c r="L77">
+        <v>2616040</v>
+      </c>
+      <c r="M77" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="78" spans="1:13">
+      <c r="A78" t="s">
+        <v>13</v>
+      </c>
+      <c r="B78" t="s">
+        <v>14</v>
+      </c>
+      <c r="C78">
+        <v>2026</v>
+      </c>
+      <c r="D78" t="s">
+        <v>15</v>
+      </c>
+      <c r="E78" t="s">
+        <v>16</v>
+      </c>
+      <c r="F78" t="s">
+        <v>17</v>
+      </c>
+      <c r="G78" t="s">
+        <v>18</v>
+      </c>
+      <c r="H78" t="s">
+        <v>95</v>
+      </c>
+      <c r="I78" t="s">
+        <v>213</v>
+      </c>
+      <c r="J78" t="s">
+        <v>324</v>
+      </c>
+      <c r="K78" t="s">
+        <v>360</v>
+      </c>
+      <c r="L78">
+        <v>273579</v>
+      </c>
+      <c r="M78" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="79" spans="1:13">
+      <c r="A79" t="s">
+        <v>13</v>
+      </c>
+      <c r="B79" t="s">
+        <v>14</v>
+      </c>
+      <c r="C79">
+        <v>2026</v>
+      </c>
+      <c r="D79" t="s">
+        <v>15</v>
+      </c>
+      <c r="E79" t="s">
+        <v>16</v>
+      </c>
+      <c r="F79" t="s">
+        <v>17</v>
+      </c>
+      <c r="G79" t="s">
+        <v>18</v>
+      </c>
+      <c r="H79" t="s">
+        <v>96</v>
+      </c>
+      <c r="I79" t="s">
+        <v>214</v>
+      </c>
+      <c r="J79" t="s">
+        <v>325</v>
+      </c>
+      <c r="K79" t="s">
+        <v>368</v>
+      </c>
+      <c r="L79">
+        <v>506123</v>
+      </c>
+      <c r="M79" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="80" spans="1:13">
+      <c r="A80" t="s">
+        <v>13</v>
+      </c>
+      <c r="B80" t="s">
+        <v>14</v>
+      </c>
+      <c r="C80">
+        <v>2026</v>
+      </c>
+      <c r="D80" t="s">
+        <v>15</v>
+      </c>
+      <c r="E80" t="s">
+        <v>16</v>
+      </c>
+      <c r="F80" t="s">
+        <v>17</v>
+      </c>
+      <c r="G80" t="s">
+        <v>18</v>
+      </c>
+      <c r="H80" t="s">
+        <v>97</v>
+      </c>
+      <c r="I80" t="s">
+        <v>215</v>
+      </c>
+      <c r="J80" t="s">
+        <v>326</v>
+      </c>
+      <c r="K80" t="s">
+        <v>369</v>
+      </c>
+      <c r="L80">
+        <v>554327</v>
+      </c>
+      <c r="M80" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="81" spans="1:13">
+      <c r="A81" t="s">
+        <v>13</v>
+      </c>
+      <c r="B81" t="s">
+        <v>14</v>
+      </c>
+      <c r="C81">
+        <v>2026</v>
+      </c>
+      <c r="D81" t="s">
+        <v>15</v>
+      </c>
+      <c r="E81" t="s">
+        <v>16</v>
+      </c>
+      <c r="F81" t="s">
+        <v>17</v>
+      </c>
+      <c r="G81" t="s">
+        <v>18</v>
+      </c>
+      <c r="H81" t="s">
+        <v>98</v>
+      </c>
+      <c r="I81" t="s">
+        <v>216</v>
+      </c>
+      <c r="J81" t="s">
+        <v>327</v>
+      </c>
+      <c r="K81" t="s">
+        <v>368</v>
+      </c>
+      <c r="L81">
+        <v>569936</v>
+      </c>
+      <c r="M81" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="82" spans="1:13">
+      <c r="A82" t="s">
+        <v>13</v>
+      </c>
+      <c r="B82" t="s">
+        <v>14</v>
+      </c>
+      <c r="C82">
+        <v>2026</v>
+      </c>
+      <c r="D82" t="s">
+        <v>15</v>
+      </c>
+      <c r="E82" t="s">
+        <v>16</v>
+      </c>
+      <c r="F82" t="s">
+        <v>17</v>
+      </c>
+      <c r="G82" t="s">
+        <v>18</v>
+      </c>
+      <c r="H82" t="s">
+        <v>99</v>
+      </c>
+      <c r="I82" t="s">
+        <v>217</v>
+      </c>
+      <c r="J82" t="s">
+        <v>327</v>
+      </c>
+      <c r="K82" t="s">
+        <v>362</v>
+      </c>
+      <c r="L82">
+        <v>513072</v>
+      </c>
+      <c r="M82" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="83" spans="1:13">
+      <c r="A83" t="s">
+        <v>13</v>
+      </c>
+      <c r="B83" t="s">
+        <v>14</v>
+      </c>
+      <c r="C83">
+        <v>2026</v>
+      </c>
+      <c r="D83" t="s">
+        <v>15</v>
+      </c>
+      <c r="E83" t="s">
+        <v>16</v>
+      </c>
+      <c r="F83" t="s">
+        <v>17</v>
+      </c>
+      <c r="G83" t="s">
+        <v>18</v>
+      </c>
+      <c r="H83" t="s">
+        <v>100</v>
+      </c>
+      <c r="I83" t="s">
+        <v>218</v>
+      </c>
+      <c r="J83" t="s">
+        <v>328</v>
+      </c>
+      <c r="K83" t="s">
+        <v>370</v>
+      </c>
+      <c r="L83">
+        <v>1852495</v>
+      </c>
+      <c r="M83" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="84" spans="1:13">
+      <c r="A84" t="s">
+        <v>13</v>
+      </c>
+      <c r="B84" t="s">
+        <v>14</v>
+      </c>
+      <c r="C84">
+        <v>2026</v>
+      </c>
+      <c r="D84" t="s">
+        <v>15</v>
+      </c>
+      <c r="E84" t="s">
+        <v>16</v>
+      </c>
+      <c r="F84" t="s">
+        <v>17</v>
+      </c>
+      <c r="G84" t="s">
+        <v>18</v>
+      </c>
+      <c r="H84" t="s">
+        <v>101</v>
+      </c>
+      <c r="I84" t="s">
+        <v>219</v>
+      </c>
+      <c r="J84" t="s">
+        <v>328</v>
+      </c>
+      <c r="K84" t="s">
+        <v>363</v>
+      </c>
+      <c r="L84">
+        <v>1514320</v>
+      </c>
+      <c r="M84" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="85" spans="1:13">
+      <c r="A85" t="s">
+        <v>13</v>
+      </c>
+      <c r="B85" t="s">
+        <v>14</v>
+      </c>
+      <c r="C85">
+        <v>2026</v>
+      </c>
+      <c r="D85" t="s">
+        <v>15</v>
+      </c>
+      <c r="E85" t="s">
+        <v>16</v>
+      </c>
+      <c r="F85" t="s">
+        <v>17</v>
+      </c>
+      <c r="G85" t="s">
+        <v>18</v>
+      </c>
+      <c r="H85" t="s">
+        <v>102</v>
+      </c>
+      <c r="I85" t="s">
+        <v>220</v>
+      </c>
+      <c r="J85" t="s">
+        <v>329</v>
+      </c>
+      <c r="K85" t="s">
+        <v>359</v>
+      </c>
+      <c r="L85">
+        <v>1258720</v>
+      </c>
+      <c r="M85" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="86" spans="1:13">
+      <c r="A86" t="s">
+        <v>13</v>
+      </c>
+      <c r="B86" t="s">
+        <v>14</v>
+      </c>
+      <c r="C86">
+        <v>2026</v>
+      </c>
+      <c r="D86" t="s">
+        <v>15</v>
+      </c>
+      <c r="E86" t="s">
+        <v>16</v>
+      </c>
+      <c r="F86" t="s">
+        <v>17</v>
+      </c>
+      <c r="G86" t="s">
+        <v>18</v>
+      </c>
+      <c r="H86" t="s">
+        <v>103</v>
+      </c>
+      <c r="I86" t="s">
+        <v>221</v>
+      </c>
+      <c r="J86" t="s">
+        <v>329</v>
+      </c>
+      <c r="K86" t="s">
+        <v>369</v>
+      </c>
+      <c r="L86">
+        <v>1176410</v>
+      </c>
+      <c r="M86" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="87" spans="1:13">
+      <c r="A87" t="s">
+        <v>13</v>
+      </c>
+      <c r="B87" t="s">
+        <v>14</v>
+      </c>
+      <c r="C87">
+        <v>2026</v>
+      </c>
+      <c r="D87" t="s">
+        <v>15</v>
+      </c>
+      <c r="E87" t="s">
+        <v>16</v>
+      </c>
+      <c r="F87" t="s">
+        <v>17</v>
+      </c>
+      <c r="G87" t="s">
+        <v>18</v>
+      </c>
+      <c r="H87" t="s">
+        <v>104</v>
+      </c>
+      <c r="I87" t="s">
+        <v>222</v>
+      </c>
+      <c r="J87" t="s">
+        <v>330</v>
+      </c>
+      <c r="K87" t="s">
+        <v>361</v>
+      </c>
+      <c r="L87">
+        <v>1301404</v>
+      </c>
+      <c r="M87" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="88" spans="1:13">
+      <c r="A88" t="s">
+        <v>13</v>
+      </c>
+      <c r="B88" t="s">
+        <v>14</v>
+      </c>
+      <c r="C88">
+        <v>2026</v>
+      </c>
+      <c r="D88" t="s">
+        <v>15</v>
+      </c>
+      <c r="E88" t="s">
+        <v>16</v>
+      </c>
+      <c r="F88" t="s">
+        <v>17</v>
+      </c>
+      <c r="G88" t="s">
+        <v>18</v>
+      </c>
+      <c r="H88" t="s">
+        <v>105</v>
+      </c>
+      <c r="I88" t="s">
+        <v>223</v>
+      </c>
+      <c r="J88" t="s">
+        <v>331</v>
+      </c>
+      <c r="K88" t="s">
+        <v>370</v>
+      </c>
+      <c r="L88">
+        <v>643482</v>
+      </c>
+      <c r="M88" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="89" spans="1:13">
+      <c r="A89" t="s">
+        <v>13</v>
+      </c>
+      <c r="B89" t="s">
+        <v>14</v>
+      </c>
+      <c r="C89">
+        <v>2026</v>
+      </c>
+      <c r="D89" t="s">
+        <v>15</v>
+      </c>
+      <c r="E89" t="s">
+        <v>16</v>
+      </c>
+      <c r="F89" t="s">
+        <v>17</v>
+      </c>
+      <c r="G89" t="s">
+        <v>18</v>
+      </c>
+      <c r="H89" t="s">
+        <v>106</v>
+      </c>
+      <c r="I89" t="s">
+        <v>224</v>
+      </c>
+      <c r="J89" t="s">
+        <v>332</v>
+      </c>
+      <c r="K89" t="s">
+        <v>360</v>
+      </c>
+      <c r="L89">
+        <v>946757</v>
+      </c>
+      <c r="M89" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="90" spans="1:13">
+      <c r="A90" t="s">
+        <v>13</v>
+      </c>
+      <c r="B90" t="s">
+        <v>14</v>
+      </c>
+      <c r="C90">
+        <v>2026</v>
+      </c>
+      <c r="D90" t="s">
+        <v>15</v>
+      </c>
+      <c r="E90" t="s">
+        <v>16</v>
+      </c>
+      <c r="F90" t="s">
+        <v>17</v>
+      </c>
+      <c r="G90" t="s">
+        <v>18</v>
+      </c>
+      <c r="H90" t="s">
+        <v>107</v>
+      </c>
+      <c r="I90" t="s">
+        <v>225</v>
+      </c>
+      <c r="J90" t="s">
+        <v>333</v>
+      </c>
+      <c r="K90" t="s">
+        <v>362</v>
+      </c>
+      <c r="L90">
+        <v>256520</v>
+      </c>
+      <c r="M90" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="91" spans="1:13">
+      <c r="A91" t="s">
+        <v>13</v>
+      </c>
+      <c r="B91" t="s">
+        <v>14</v>
+      </c>
+      <c r="C91">
+        <v>2026</v>
+      </c>
+      <c r="D91" t="s">
+        <v>15</v>
+      </c>
+      <c r="E91" t="s">
+        <v>16</v>
+      </c>
+      <c r="F91" t="s">
+        <v>17</v>
+      </c>
+      <c r="G91" t="s">
+        <v>18</v>
+      </c>
+      <c r="H91" t="s">
+        <v>108</v>
+      </c>
+      <c r="I91" t="s">
+        <v>226</v>
+      </c>
+      <c r="J91" t="s">
+        <v>334</v>
+      </c>
+      <c r="K91" t="s">
+        <v>362</v>
+      </c>
+      <c r="L91">
+        <v>484020</v>
+      </c>
+      <c r="M91" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="92" spans="1:13">
+      <c r="A92" t="s">
+        <v>13</v>
+      </c>
+      <c r="B92" t="s">
+        <v>14</v>
+      </c>
+      <c r="C92">
+        <v>2026</v>
+      </c>
+      <c r="D92" t="s">
+        <v>15</v>
+      </c>
+      <c r="E92" t="s">
+        <v>16</v>
+      </c>
+      <c r="F92" t="s">
+        <v>17</v>
+      </c>
+      <c r="G92" t="s">
+        <v>18</v>
+      </c>
+      <c r="H92" t="s">
+        <v>109</v>
+      </c>
+      <c r="I92" t="s">
+        <v>227</v>
+      </c>
+      <c r="J92" t="s">
+        <v>335</v>
+      </c>
+      <c r="K92" t="s">
+        <v>361</v>
+      </c>
+      <c r="L92">
+        <v>648268</v>
+      </c>
+      <c r="M92" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="93" spans="1:13">
+      <c r="A93" t="s">
+        <v>13</v>
+      </c>
+      <c r="B93" t="s">
+        <v>14</v>
+      </c>
+      <c r="C93">
+        <v>2026</v>
+      </c>
+      <c r="D93" t="s">
+        <v>15</v>
+      </c>
+      <c r="E93" t="s">
+        <v>16</v>
+      </c>
+      <c r="F93" t="s">
+        <v>17</v>
+      </c>
+      <c r="G93" t="s">
+        <v>18</v>
+      </c>
+      <c r="H93" t="s">
+        <v>110</v>
+      </c>
+      <c r="I93" t="s">
+        <v>228</v>
+      </c>
+      <c r="J93" t="s">
+        <v>336</v>
+      </c>
+      <c r="K93" t="s">
+        <v>368</v>
+      </c>
+      <c r="L93">
+        <v>2036492</v>
+      </c>
+      <c r="M93" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="94" spans="1:13">
+      <c r="A94" t="s">
+        <v>13</v>
+      </c>
+      <c r="B94" t="s">
+        <v>14</v>
+      </c>
+      <c r="C94">
+        <v>2026</v>
+      </c>
+      <c r="D94" t="s">
+        <v>15</v>
+      </c>
+      <c r="E94" t="s">
+        <v>16</v>
+      </c>
+      <c r="F94" t="s">
+        <v>17</v>
+      </c>
+      <c r="G94" t="s">
+        <v>18</v>
+      </c>
+      <c r="H94" t="s">
+        <v>111</v>
+      </c>
+      <c r="I94" t="s">
+        <v>229</v>
+      </c>
+      <c r="J94" t="s">
+        <v>336</v>
+      </c>
+      <c r="K94" t="s">
+        <v>362</v>
+      </c>
+      <c r="L94">
+        <v>1372944</v>
+      </c>
+      <c r="M94" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="95" spans="1:13">
+      <c r="A95" t="s">
+        <v>13</v>
+      </c>
+      <c r="B95" t="s">
+        <v>14</v>
+      </c>
+      <c r="C95">
+        <v>2026</v>
+      </c>
+      <c r="D95" t="s">
+        <v>15</v>
+      </c>
+      <c r="E95" t="s">
+        <v>16</v>
+      </c>
+      <c r="F95" t="s">
+        <v>17</v>
+      </c>
+      <c r="G95" t="s">
+        <v>18</v>
+      </c>
+      <c r="H95" t="s">
+        <v>112</v>
+      </c>
+      <c r="I95" t="s">
+        <v>230</v>
+      </c>
+      <c r="J95" t="s">
+        <v>336</v>
+      </c>
+      <c r="K95" t="s">
+        <v>367</v>
+      </c>
+      <c r="L95">
+        <v>2215016</v>
+      </c>
+      <c r="M95" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="96" spans="1:13">
+      <c r="A96" t="s">
+        <v>13</v>
+      </c>
+      <c r="B96" t="s">
+        <v>14</v>
+      </c>
+      <c r="C96">
+        <v>2026</v>
+      </c>
+      <c r="D96" t="s">
+        <v>15</v>
+      </c>
+      <c r="E96" t="s">
+        <v>16</v>
+      </c>
+      <c r="F96" t="s">
+        <v>17</v>
+      </c>
+      <c r="G96" t="s">
+        <v>18</v>
+      </c>
+      <c r="H96" t="s">
+        <v>113</v>
+      </c>
+      <c r="I96" t="s">
+        <v>231</v>
+      </c>
+      <c r="J96" t="s">
+        <v>337</v>
+      </c>
+      <c r="K96" t="s">
+        <v>370</v>
+      </c>
+      <c r="L96">
+        <v>3273093</v>
+      </c>
+      <c r="M96" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="97" spans="1:13">
+      <c r="A97" t="s">
+        <v>13</v>
+      </c>
+      <c r="B97" t="s">
+        <v>14</v>
+      </c>
+      <c r="C97">
+        <v>2026</v>
+      </c>
+      <c r="D97" t="s">
+        <v>15</v>
+      </c>
+      <c r="E97" t="s">
+        <v>16</v>
+      </c>
+      <c r="F97" t="s">
+        <v>17</v>
+      </c>
+      <c r="G97" t="s">
+        <v>18</v>
+      </c>
+      <c r="H97" t="s">
+        <v>114</v>
+      </c>
+      <c r="I97" t="s">
+        <v>232</v>
+      </c>
+      <c r="J97" t="s">
+        <v>338</v>
+      </c>
+      <c r="K97" t="s">
+        <v>367</v>
+      </c>
+      <c r="L97">
+        <v>585486</v>
+      </c>
+      <c r="M97" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="98" spans="1:13">
+      <c r="A98" t="s">
+        <v>13</v>
+      </c>
+      <c r="B98" t="s">
+        <v>14</v>
+      </c>
+      <c r="C98">
+        <v>2026</v>
+      </c>
+      <c r="D98" t="s">
+        <v>15</v>
+      </c>
+      <c r="E98" t="s">
+        <v>16</v>
+      </c>
+      <c r="F98" t="s">
+        <v>17</v>
+      </c>
+      <c r="G98" t="s">
+        <v>18</v>
+      </c>
+      <c r="H98" t="s">
+        <v>115</v>
+      </c>
+      <c r="I98" t="s">
+        <v>233</v>
+      </c>
+      <c r="J98" t="s">
+        <v>339</v>
+      </c>
+      <c r="K98" t="s">
+        <v>359</v>
+      </c>
+      <c r="L98">
+        <v>557982</v>
+      </c>
+      <c r="M98" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="99" spans="1:13">
+      <c r="A99" t="s">
+        <v>13</v>
+      </c>
+      <c r="B99" t="s">
+        <v>14</v>
+      </c>
+      <c r="C99">
+        <v>2026</v>
+      </c>
+      <c r="D99" t="s">
+        <v>15</v>
+      </c>
+      <c r="E99" t="s">
+        <v>16</v>
+      </c>
+      <c r="F99" t="s">
+        <v>17</v>
+      </c>
+      <c r="G99" t="s">
+        <v>18</v>
+      </c>
+      <c r="H99" t="s">
+        <v>116</v>
+      </c>
+      <c r="I99" t="s">
+        <v>234</v>
+      </c>
+      <c r="J99" t="s">
+        <v>340</v>
+      </c>
+      <c r="K99" t="s">
+        <v>364</v>
+      </c>
+      <c r="L99">
+        <v>4016944</v>
+      </c>
+      <c r="M99" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="100" spans="1:13">
+      <c r="A100" t="s">
+        <v>13</v>
+      </c>
+      <c r="B100" t="s">
+        <v>14</v>
+      </c>
+      <c r="C100">
+        <v>2026</v>
+      </c>
+      <c r="D100" t="s">
+        <v>15</v>
+      </c>
+      <c r="E100" t="s">
+        <v>16</v>
+      </c>
+      <c r="F100" t="s">
+        <v>17</v>
+      </c>
+      <c r="G100" t="s">
+        <v>18</v>
+      </c>
+      <c r="H100" t="s">
+        <v>117</v>
+      </c>
+      <c r="I100" t="s">
+        <v>235</v>
+      </c>
+      <c r="J100" t="s">
+        <v>341</v>
+      </c>
+      <c r="K100" t="s">
+        <v>363</v>
+      </c>
+      <c r="L100">
+        <v>2850510</v>
+      </c>
+      <c r="M100" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="101" spans="1:13">
+      <c r="A101" t="s">
+        <v>13</v>
+      </c>
+      <c r="B101" t="s">
+        <v>14</v>
+      </c>
+      <c r="C101">
+        <v>2026</v>
+      </c>
+      <c r="D101" t="s">
+        <v>15</v>
+      </c>
+      <c r="E101" t="s">
+        <v>16</v>
+      </c>
+      <c r="F101" t="s">
+        <v>17</v>
+      </c>
+      <c r="G101" t="s">
+        <v>18</v>
+      </c>
+      <c r="H101" t="s">
+        <v>118</v>
+      </c>
+      <c r="I101" t="s">
+        <v>236</v>
+      </c>
+      <c r="J101" t="s">
+        <v>342</v>
+      </c>
+      <c r="K101" t="s">
+        <v>367</v>
+      </c>
+      <c r="L101">
+        <v>1172972</v>
+      </c>
+      <c r="M101" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="102" spans="1:13">
+      <c r="A102" t="s">
+        <v>13</v>
+      </c>
+      <c r="B102" t="s">
+        <v>14</v>
+      </c>
+      <c r="C102">
+        <v>2026</v>
+      </c>
+      <c r="D102" t="s">
+        <v>15</v>
+      </c>
+      <c r="E102" t="s">
+        <v>16</v>
+      </c>
+      <c r="F102" t="s">
+        <v>17</v>
+      </c>
+      <c r="G102" t="s">
+        <v>18</v>
+      </c>
+      <c r="H102" t="s">
+        <v>119</v>
+      </c>
+      <c r="I102" t="s">
+        <v>237</v>
+      </c>
+      <c r="J102" t="s">
+        <v>342</v>
+      </c>
+      <c r="K102" t="s">
+        <v>360</v>
+      </c>
+      <c r="L102">
+        <v>1016660</v>
+      </c>
+      <c r="M102" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="103" spans="1:13">
+      <c r="A103" t="s">
+        <v>13</v>
+      </c>
+      <c r="B103" t="s">
+        <v>14</v>
+      </c>
+      <c r="C103">
+        <v>2026</v>
+      </c>
+      <c r="D103" t="s">
+        <v>15</v>
+      </c>
+      <c r="E103" t="s">
+        <v>16</v>
+      </c>
+      <c r="F103" t="s">
+        <v>17</v>
+      </c>
+      <c r="G103" t="s">
+        <v>18</v>
+      </c>
+      <c r="H103" t="s">
+        <v>120</v>
+      </c>
+      <c r="I103" t="s">
+        <v>238</v>
+      </c>
+      <c r="J103" t="s">
+        <v>343</v>
+      </c>
+      <c r="K103" t="s">
+        <v>360</v>
+      </c>
+      <c r="L103">
+        <v>956502</v>
+      </c>
+      <c r="M103" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="104" spans="1:13">
+      <c r="A104" t="s">
+        <v>13</v>
+      </c>
+      <c r="B104" t="s">
+        <v>14</v>
+      </c>
+      <c r="C104">
+        <v>2026</v>
+      </c>
+      <c r="D104" t="s">
+        <v>15</v>
+      </c>
+      <c r="E104" t="s">
+        <v>16</v>
+      </c>
+      <c r="F104" t="s">
+        <v>17</v>
+      </c>
+      <c r="G104" t="s">
+        <v>18</v>
+      </c>
+      <c r="H104" t="s">
+        <v>121</v>
+      </c>
+      <c r="I104" t="s">
+        <v>239</v>
+      </c>
+      <c r="J104" t="s">
+        <v>344</v>
+      </c>
+      <c r="K104" t="s">
+        <v>359</v>
+      </c>
+      <c r="L104">
+        <v>522793</v>
+      </c>
+      <c r="M104" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="105" spans="1:13">
+      <c r="A105" t="s">
+        <v>13</v>
+      </c>
+      <c r="B105" t="s">
+        <v>14</v>
+      </c>
+      <c r="C105">
+        <v>2026</v>
+      </c>
+      <c r="D105" t="s">
+        <v>15</v>
+      </c>
+      <c r="E105" t="s">
+        <v>16</v>
+      </c>
+      <c r="F105" t="s">
+        <v>17</v>
+      </c>
+      <c r="G105" t="s">
+        <v>18</v>
+      </c>
+      <c r="H105" t="s">
+        <v>122</v>
+      </c>
+      <c r="I105" t="s">
+        <v>240</v>
+      </c>
+      <c r="J105" t="s">
+        <v>345</v>
+      </c>
+      <c r="K105" t="s">
+        <v>363</v>
+      </c>
+      <c r="L105">
+        <v>751376</v>
+      </c>
+      <c r="M105" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="106" spans="1:13">
+      <c r="A106" t="s">
+        <v>13</v>
+      </c>
+      <c r="B106" t="s">
+        <v>14</v>
+      </c>
+      <c r="C106">
+        <v>2026</v>
+      </c>
+      <c r="D106" t="s">
+        <v>15</v>
+      </c>
+      <c r="E106" t="s">
+        <v>16</v>
+      </c>
+      <c r="F106" t="s">
+        <v>17</v>
+      </c>
+      <c r="G106" t="s">
+        <v>18</v>
+      </c>
+      <c r="H106" t="s">
+        <v>123</v>
+      </c>
+      <c r="I106" t="s">
+        <v>241</v>
+      </c>
+      <c r="J106" t="s">
+        <v>345</v>
+      </c>
+      <c r="K106" t="s">
+        <v>362</v>
+      </c>
+      <c r="L106">
+        <v>681304</v>
+      </c>
+      <c r="M106" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="107" spans="1:13">
+      <c r="A107" t="s">
+        <v>13</v>
+      </c>
+      <c r="B107" t="s">
+        <v>14</v>
+      </c>
+      <c r="C107">
+        <v>2026</v>
+      </c>
+      <c r="D107" t="s">
+        <v>15</v>
+      </c>
+      <c r="E107" t="s">
+        <v>16</v>
+      </c>
+      <c r="F107" t="s">
+        <v>17</v>
+      </c>
+      <c r="G107" t="s">
+        <v>18</v>
+      </c>
+      <c r="H107" t="s">
+        <v>124</v>
+      </c>
+      <c r="I107" t="s">
+        <v>242</v>
+      </c>
+      <c r="J107" t="s">
+        <v>346</v>
+      </c>
+      <c r="K107" t="s">
+        <v>359</v>
+      </c>
+      <c r="L107">
+        <v>557982</v>
+      </c>
+      <c r="M107" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="108" spans="1:13">
+      <c r="A108" t="s">
+        <v>13</v>
+      </c>
+      <c r="B108" t="s">
+        <v>14</v>
+      </c>
+      <c r="C108">
+        <v>2026</v>
+      </c>
+      <c r="D108" t="s">
+        <v>15</v>
+      </c>
+      <c r="E108" t="s">
+        <v>16</v>
+      </c>
+      <c r="F108" t="s">
+        <v>17</v>
+      </c>
+      <c r="G108" t="s">
+        <v>18</v>
+      </c>
+      <c r="H108" t="s">
+        <v>125</v>
+      </c>
+      <c r="I108" t="s">
+        <v>243</v>
+      </c>
+      <c r="J108" t="s">
+        <v>347</v>
+      </c>
+      <c r="K108" t="s">
+        <v>359</v>
+      </c>
+      <c r="L108">
+        <v>593026</v>
+      </c>
+      <c r="M108" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="109" spans="1:13">
+      <c r="A109" t="s">
+        <v>13</v>
+      </c>
+      <c r="B109" t="s">
+        <v>14</v>
+      </c>
+      <c r="C109">
+        <v>2026</v>
+      </c>
+      <c r="D109" t="s">
+        <v>15</v>
+      </c>
+      <c r="E109" t="s">
+        <v>16</v>
+      </c>
+      <c r="F109" t="s">
+        <v>17</v>
+      </c>
+      <c r="G109" t="s">
+        <v>18</v>
+      </c>
+      <c r="H109" t="s">
+        <v>126</v>
+      </c>
+      <c r="I109" t="s">
+        <v>244</v>
+      </c>
+      <c r="J109" t="s">
+        <v>348</v>
+      </c>
+      <c r="K109" t="s">
+        <v>363</v>
+      </c>
+      <c r="L109">
+        <v>3295132</v>
+      </c>
+      <c r="M109" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="110" spans="1:13">
+      <c r="A110" t="s">
+        <v>13</v>
+      </c>
+      <c r="B110" t="s">
+        <v>14</v>
+      </c>
+      <c r="C110">
+        <v>2026</v>
+      </c>
+      <c r="D110" t="s">
+        <v>15</v>
+      </c>
+      <c r="E110" t="s">
+        <v>16</v>
+      </c>
+      <c r="F110" t="s">
+        <v>17</v>
+      </c>
+      <c r="G110" t="s">
+        <v>18</v>
+      </c>
+      <c r="H110" t="s">
+        <v>127</v>
+      </c>
+      <c r="I110" t="s">
+        <v>245</v>
+      </c>
+      <c r="J110" t="s">
+        <v>349</v>
+      </c>
+      <c r="K110" t="s">
+        <v>361</v>
+      </c>
+      <c r="L110">
+        <v>650772</v>
+      </c>
+      <c r="M110" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="111" spans="1:13">
+      <c r="A111" t="s">
+        <v>13</v>
+      </c>
+      <c r="B111" t="s">
+        <v>14</v>
+      </c>
+      <c r="C111">
+        <v>2026</v>
+      </c>
+      <c r="D111" t="s">
+        <v>15</v>
+      </c>
+      <c r="E111" t="s">
+        <v>16</v>
+      </c>
+      <c r="F111" t="s">
+        <v>17</v>
+      </c>
+      <c r="G111" t="s">
+        <v>18</v>
+      </c>
+      <c r="H111" t="s">
+        <v>128</v>
+      </c>
+      <c r="I111" t="s">
+        <v>246</v>
+      </c>
+      <c r="J111" t="s">
+        <v>350</v>
+      </c>
+      <c r="K111" t="s">
+        <v>368</v>
+      </c>
+      <c r="L111">
+        <v>506123</v>
+      </c>
+      <c r="M111" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="112" spans="1:13">
+      <c r="A112" t="s">
+        <v>13</v>
+      </c>
+      <c r="B112" t="s">
+        <v>14</v>
+      </c>
+      <c r="C112">
+        <v>2026</v>
+      </c>
+      <c r="D112" t="s">
+        <v>15</v>
+      </c>
+      <c r="E112" t="s">
+        <v>16</v>
+      </c>
+      <c r="F112" t="s">
+        <v>17</v>
+      </c>
+      <c r="G112" t="s">
+        <v>18</v>
+      </c>
+      <c r="H112" t="s">
+        <v>129</v>
+      </c>
+      <c r="I112" t="s">
+        <v>247</v>
+      </c>
+      <c r="J112" t="s">
+        <v>351</v>
+      </c>
+      <c r="K112" t="s">
+        <v>359</v>
+      </c>
+      <c r="L112">
+        <v>1574379</v>
+      </c>
+      <c r="M112" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="113" spans="1:13">
+      <c r="A113" t="s">
+        <v>13</v>
+      </c>
+      <c r="B113" t="s">
+        <v>14</v>
+      </c>
+      <c r="C113">
+        <v>2026</v>
+      </c>
+      <c r="D113" t="s">
+        <v>15</v>
+      </c>
+      <c r="E113" t="s">
+        <v>16</v>
+      </c>
+      <c r="F113" t="s">
+        <v>17</v>
+      </c>
+      <c r="G113" t="s">
+        <v>18</v>
+      </c>
+      <c r="H113" t="s">
+        <v>130</v>
+      </c>
+      <c r="I113" t="s">
+        <v>248</v>
+      </c>
+      <c r="J113" t="s">
+        <v>352</v>
+      </c>
+      <c r="K113" t="s">
+        <v>360</v>
+      </c>
+      <c r="L113">
+        <v>444757</v>
+      </c>
+      <c r="M113" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="114" spans="1:13">
+      <c r="A114" t="s">
+        <v>13</v>
+      </c>
+      <c r="B114" t="s">
+        <v>14</v>
+      </c>
+      <c r="C114">
+        <v>2026</v>
+      </c>
+      <c r="D114" t="s">
+        <v>15</v>
+      </c>
+      <c r="E114" t="s">
+        <v>16</v>
+      </c>
+      <c r="F114" t="s">
+        <v>17</v>
+      </c>
+      <c r="G114" t="s">
+        <v>18</v>
+      </c>
+      <c r="H114" t="s">
+        <v>131</v>
+      </c>
+      <c r="I114" t="s">
+        <v>249</v>
+      </c>
+      <c r="J114" t="s">
+        <v>353</v>
+      </c>
+      <c r="K114" t="s">
+        <v>367</v>
+      </c>
+      <c r="L114">
+        <v>3654161</v>
+      </c>
+      <c r="M114" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="115" spans="1:13">
+      <c r="A115" t="s">
+        <v>13</v>
+      </c>
+      <c r="B115" t="s">
+        <v>14</v>
+      </c>
+      <c r="C115">
+        <v>2026</v>
+      </c>
+      <c r="D115" t="s">
+        <v>15</v>
+      </c>
+      <c r="E115" t="s">
+        <v>16</v>
+      </c>
+      <c r="F115" t="s">
+        <v>17</v>
+      </c>
+      <c r="G115" t="s">
+        <v>18</v>
+      </c>
+      <c r="H115" t="s">
+        <v>132</v>
+      </c>
+      <c r="I115" t="s">
+        <v>250</v>
+      </c>
+      <c r="J115" t="s">
+        <v>354</v>
+      </c>
+      <c r="K115" t="s">
+        <v>360</v>
+      </c>
+      <c r="L115">
+        <v>956502</v>
+      </c>
+      <c r="M115" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="116" spans="1:13">
+      <c r="A116" t="s">
+        <v>13</v>
+      </c>
+      <c r="B116" t="s">
+        <v>14</v>
+      </c>
+      <c r="C116">
+        <v>2026</v>
+      </c>
+      <c r="D116" t="s">
+        <v>15</v>
+      </c>
+      <c r="E116" t="s">
+        <v>16</v>
+      </c>
+      <c r="F116" t="s">
+        <v>17</v>
+      </c>
+      <c r="G116" t="s">
+        <v>18</v>
+      </c>
+      <c r="H116" t="s">
+        <v>133</v>
+      </c>
+      <c r="I116" t="s">
+        <v>251</v>
+      </c>
+      <c r="J116" t="s">
+        <v>355</v>
+      </c>
+      <c r="K116" t="s">
+        <v>359</v>
+      </c>
+      <c r="L116">
+        <v>343171</v>
+      </c>
+      <c r="M116" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="117" spans="1:13">
+      <c r="A117" t="s">
+        <v>13</v>
+      </c>
+      <c r="B117" t="s">
+        <v>14</v>
+      </c>
+      <c r="C117">
+        <v>2026</v>
+      </c>
+      <c r="D117" t="s">
+        <v>15</v>
+      </c>
+      <c r="E117" t="s">
+        <v>16</v>
+      </c>
+      <c r="F117" t="s">
+        <v>17</v>
+      </c>
+      <c r="G117" t="s">
+        <v>18</v>
+      </c>
+      <c r="H117" t="s">
+        <v>134</v>
+      </c>
+      <c r="I117" t="s">
+        <v>252</v>
+      </c>
+      <c r="J117" t="s">
+        <v>356</v>
+      </c>
+      <c r="K117" t="s">
+        <v>361</v>
+      </c>
+      <c r="L117">
+        <v>577752</v>
+      </c>
+      <c r="M117" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="118" spans="1:13">
+      <c r="A118" t="s">
+        <v>13</v>
+      </c>
+      <c r="B118" t="s">
+        <v>14</v>
+      </c>
+      <c r="C118">
+        <v>2026</v>
+      </c>
+      <c r="D118" t="s">
+        <v>15</v>
+      </c>
+      <c r="E118" t="s">
+        <v>16</v>
+      </c>
+      <c r="F118" t="s">
+        <v>17</v>
+      </c>
+      <c r="G118" t="s">
+        <v>18</v>
+      </c>
+      <c r="H118" t="s">
+        <v>135</v>
+      </c>
+      <c r="I118" t="s">
+        <v>253</v>
+      </c>
+      <c r="J118" t="s">
+        <v>357</v>
+      </c>
+      <c r="K118" t="s">
+        <v>364</v>
+      </c>
+      <c r="L118">
+        <v>665127</v>
+      </c>
+      <c r="M118" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="119" spans="1:13">
+      <c r="A119" t="s">
+        <v>13</v>
+      </c>
+      <c r="B119" t="s">
+        <v>14</v>
+      </c>
+      <c r="C119">
+        <v>2026</v>
+      </c>
+      <c r="D119" t="s">
+        <v>15</v>
+      </c>
+      <c r="E119" t="s">
+        <v>16</v>
+      </c>
+      <c r="F119" t="s">
+        <v>17</v>
+      </c>
+      <c r="G119" t="s">
+        <v>18</v>
+      </c>
+      <c r="H119" t="s">
+        <v>136</v>
+      </c>
+      <c r="I119" t="s">
+        <v>254</v>
+      </c>
+      <c r="J119" t="s">
+        <v>358</v>
+      </c>
+      <c r="K119" t="s">
+        <v>361</v>
+      </c>
+      <c r="L119">
+        <v>614324</v>
+      </c>
+      <c r="M119" t="s">
+        <v>371</v>
       </c>
     </row>
   </sheetData>

</xml_diff>